<commit_message>
Updated STTI latest value
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -734,7 +734,7 @@
         <v>4.2</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1.162</v>
+        <v>1.14</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>0.82</v>
@@ -770,7 +770,7 @@
         <v>4.2</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1.162</v>
+        <v>1.14</v>
       </c>
       <c r="G3" s="7" t="n">
         <v>0.82</v>
@@ -806,7 +806,7 @@
         <v>4.2</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>1.162</v>
+        <v>1.14</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>0.82</v>
@@ -842,7 +842,7 @@
         <v>4.2</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1.162</v>
+        <v>1.14</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>0.82</v>
@@ -878,7 +878,7 @@
         <v>4.2</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>1.162</v>
+        <v>1.14</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0.82</v>
@@ -914,7 +914,7 @@
         <v>4.2</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1.162</v>
+        <v>1.14</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>0.82</v>
@@ -950,7 +950,7 @@
         <v>4.2</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>1.162</v>
+        <v>1.14</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0.82</v>
@@ -986,7 +986,7 @@
         <v>4.2</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.162</v>
+        <v>1.14</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>0.82</v>
@@ -1022,7 +1022,7 @@
         <v>4.2</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1.162</v>
+        <v>1.14</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>0.82</v>
@@ -1058,7 +1058,7 @@
         <v>4.2</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1.162</v>
+        <v>1.14</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>0.82</v>
@@ -1388,7 +1388,7 @@
         </is>
       </c>
       <c r="AB2" s="4" t="n">
-        <v>295</v>
+        <v>6</v>
       </c>
       <c r="AC2" s="4" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
         </is>
       </c>
       <c r="AB3" s="7" t="n">
-        <v>6</v>
+        <v>295</v>
       </c>
       <c r="AC3" s="7" t="inlineStr">
         <is>
@@ -1722,7 +1722,7 @@
         </is>
       </c>
       <c r="AB6" s="4" t="n">
-        <v>162</v>
+        <v>5</v>
       </c>
       <c r="AC6" s="4" t="inlineStr">
         <is>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="AB7" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AC7" s="7" t="inlineStr">
         <is>
@@ -1892,7 +1892,7 @@
         </is>
       </c>
       <c r="AB8" s="4" t="n">
-        <v>8</v>
+        <v>162</v>
       </c>
       <c r="AC8" s="4" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
         <v>1</v>
       </c>
       <c r="X10" s="4" t="n">
-        <v>73</v>
+        <v>3</v>
       </c>
       <c r="Y10" s="4" t="inlineStr">
         <is>
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="X11" s="7" t="n">
-        <v>3</v>
+        <v>73</v>
       </c>
       <c r="Y11" s="7" t="inlineStr">
         <is>
@@ -2440,7 +2440,7 @@
         <v>1</v>
       </c>
       <c r="X15" s="7" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="Y15" s="7" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         <v>55</v>
       </c>
       <c r="X16" s="4" t="n">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="Y16" s="4" t="inlineStr">
         <is>
@@ -2558,7 +2558,7 @@
         <v>5519</v>
       </c>
       <c r="X17" s="7" t="n">
-        <v>77</v>
+        <v>8</v>
       </c>
       <c r="Y17" s="7" t="inlineStr">
         <is>
@@ -2617,7 +2617,7 @@
         <v>5569</v>
       </c>
       <c r="X18" s="4" t="n">
-        <v>8</v>
+        <v>77</v>
       </c>
       <c r="Y18" s="4" t="inlineStr">
         <is>
@@ -2676,7 +2676,7 @@
         <v>5621</v>
       </c>
       <c r="X19" s="7" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="Y19" s="7" t="inlineStr">
         <is>
@@ -2735,7 +2735,7 @@
         <v>5557</v>
       </c>
       <c r="X20" s="4" t="n">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="Y20" s="4" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
         </is>
       </c>
       <c r="AB20" s="4" t="n">
-        <v>327</v>
+        <v>4</v>
       </c>
       <c r="AC20" s="4" t="inlineStr">
         <is>
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="AB21" s="7" t="n">
-        <v>1</v>
+        <v>327</v>
       </c>
       <c r="AC21" s="7" t="inlineStr">
         <is>
@@ -2866,7 +2866,7 @@
         </is>
       </c>
       <c r="AB22" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AC22" s="4" t="inlineStr">
         <is>
@@ -2912,7 +2912,7 @@
         <v>5687</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="Y23" s="7" t="inlineStr">
         <is>
@@ -2925,7 +2925,7 @@
         </is>
       </c>
       <c r="AB23" s="7" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="AC23" s="7" t="inlineStr">
         <is>
@@ -2971,7 +2971,7 @@
         <v>5395</v>
       </c>
       <c r="X24" s="4" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="Y24" s="4" t="inlineStr">
         <is>
@@ -2984,7 +2984,7 @@
         </is>
       </c>
       <c r="AB24" s="4" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="AC24" s="4" t="inlineStr">
         <is>
@@ -3030,7 +3030,7 @@
         <v>5472</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="Y25" s="7" t="inlineStr">
         <is>
@@ -3043,7 +3043,7 @@
         </is>
       </c>
       <c r="AB25" s="7" t="n">
-        <v>2</v>
+        <v>155</v>
       </c>
       <c r="AC25" s="7" t="inlineStr">
         <is>
@@ -3089,7 +3089,7 @@
         <v>5687</v>
       </c>
       <c r="X26" s="4" t="n">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="Y26" s="4" t="inlineStr">
         <is>
@@ -3102,7 +3102,7 @@
         </is>
       </c>
       <c r="AB26" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AC26" s="4" t="inlineStr">
         <is>
@@ -3161,7 +3161,7 @@
         </is>
       </c>
       <c r="AB27" s="7" t="n">
-        <v>155</v>
+        <v>3</v>
       </c>
       <c r="AC27" s="7" t="inlineStr">
         <is>
@@ -3220,7 +3220,7 @@
         </is>
       </c>
       <c r="AB28" s="4" t="n">
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="AC28" s="4" t="inlineStr">
         <is>
@@ -3279,7 +3279,7 @@
         </is>
       </c>
       <c r="AB29" s="7" t="n">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="AC29" s="7" t="inlineStr">
         <is>
@@ -3812,7 +3812,7 @@
         <v>15396</v>
       </c>
       <c r="X40" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Y40" s="4" t="inlineStr">
         <is>
@@ -3853,7 +3853,7 @@
         <v>15713</v>
       </c>
       <c r="X41" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y41" s="7" t="inlineStr">
         <is>
@@ -3894,7 +3894,7 @@
         <v>14823</v>
       </c>
       <c r="X42" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Y42" s="4" t="inlineStr">
         <is>
@@ -3907,7 +3907,7 @@
         </is>
       </c>
       <c r="AB42" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AC42" s="4" t="inlineStr">
         <is>
@@ -3935,7 +3935,7 @@
         <v>14680</v>
       </c>
       <c r="X43" s="7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="Y43" s="7" t="inlineStr">
         <is>
@@ -3989,7 +3989,7 @@
         </is>
       </c>
       <c r="AB44" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="AC44" s="4" t="inlineStr">
         <is>
@@ -4058,7 +4058,7 @@
         <v>86030</v>
       </c>
       <c r="X46" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Y46" s="4" t="inlineStr">
         <is>
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="AB46" s="4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AC46" s="4" t="inlineStr">
         <is>
@@ -4099,7 +4099,7 @@
         <v>82667</v>
       </c>
       <c r="X47" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Y47" s="7" t="inlineStr">
         <is>
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="AB47" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AC47" s="7" t="inlineStr">
         <is>
@@ -4317,7 +4317,7 @@
         </is>
       </c>
       <c r="AB52" s="4" t="n">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="AC52" s="4" t="inlineStr">
         <is>
@@ -4358,7 +4358,7 @@
         </is>
       </c>
       <c r="AB53" s="7" t="n">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="AC53" s="7" t="inlineStr">
         <is>
@@ -4399,7 +4399,7 @@
         </is>
       </c>
       <c r="AB54" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC54" s="4" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
         <v>717</v>
       </c>
       <c r="X61" s="7" t="n">
-        <v>2</v>
+        <v>54</v>
       </c>
       <c r="Y61" s="7" t="inlineStr">
         <is>
@@ -4714,7 +4714,7 @@
         <v>753</v>
       </c>
       <c r="X62" s="4" t="n">
-        <v>54</v>
+        <v>2</v>
       </c>
       <c r="Y62" s="4" t="inlineStr">
         <is>
@@ -4768,7 +4768,7 @@
         </is>
       </c>
       <c r="AB63" s="7" t="n">
-        <v>1</v>
+        <v>316</v>
       </c>
       <c r="AC63" s="7" t="inlineStr">
         <is>
@@ -4809,7 +4809,7 @@
         </is>
       </c>
       <c r="AB64" s="4" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="AC64" s="4" t="inlineStr">
         <is>
@@ -4850,7 +4850,7 @@
         </is>
       </c>
       <c r="AB65" s="7" t="n">
-        <v>316</v>
+        <v>9</v>
       </c>
       <c r="AC65" s="7" t="inlineStr">
         <is>
@@ -5096,7 +5096,7 @@
         </is>
       </c>
       <c r="AB71" s="7" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AC71" s="7" t="inlineStr">
         <is>
@@ -5178,7 +5178,7 @@
         </is>
       </c>
       <c r="AB73" s="7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AC73" s="7" t="inlineStr">
         <is>
@@ -5219,7 +5219,7 @@
         </is>
       </c>
       <c r="AB74" s="4" t="n">
-        <v>1</v>
+        <v>47</v>
       </c>
       <c r="AC74" s="4" t="inlineStr">
         <is>
@@ -5260,7 +5260,7 @@
         </is>
       </c>
       <c r="AB75" s="7" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="AC75" s="7" t="inlineStr">
         <is>
@@ -5411,7 +5411,7 @@
         <v>51004</v>
       </c>
       <c r="X79" s="7" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="Y79" s="7" t="inlineStr">
         <is>
@@ -5452,7 +5452,7 @@
         <v>50744</v>
       </c>
       <c r="X80" s="4" t="n">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="Y80" s="4" t="inlineStr">
         <is>
@@ -5616,7 +5616,7 @@
         <v>49774</v>
       </c>
       <c r="X84" s="4" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="Y84" s="4" t="inlineStr">
         <is>
@@ -5629,7 +5629,7 @@
         </is>
       </c>
       <c r="AB84" s="4" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="AC84" s="4" t="inlineStr">
         <is>
@@ -5657,7 +5657,7 @@
         <v>49626</v>
       </c>
       <c r="X85" s="7" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="Y85" s="7" t="inlineStr">
         <is>
@@ -5670,7 +5670,7 @@
         </is>
       </c>
       <c r="AB85" s="7" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AC85" s="7" t="inlineStr">
         <is>
@@ -5711,7 +5711,7 @@
         </is>
       </c>
       <c r="AB86" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="AC86" s="4" t="inlineStr">
         <is>
@@ -5752,7 +5752,7 @@
         </is>
       </c>
       <c r="AB87" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AC87" s="7" t="inlineStr">
         <is>
@@ -5862,7 +5862,7 @@
         <v>1</v>
       </c>
       <c r="X90" s="4" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="Y90" s="4" t="inlineStr">
         <is>
@@ -5875,7 +5875,7 @@
         </is>
       </c>
       <c r="AB90" s="4" t="n">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="AC90" s="4" t="inlineStr">
         <is>
@@ -5903,7 +5903,7 @@
         <v>11599</v>
       </c>
       <c r="X91" s="7" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="Y91" s="7" t="inlineStr">
         <is>
@@ -5916,7 +5916,7 @@
         </is>
       </c>
       <c r="AB91" s="7" t="n">
-        <v>6</v>
+        <v>67</v>
       </c>
       <c r="AC91" s="7" t="inlineStr">
         <is>
@@ -5944,7 +5944,7 @@
         <v>11522</v>
       </c>
       <c r="X92" s="4" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="Y92" s="4" t="inlineStr">
         <is>
@@ -5957,7 +5957,7 @@
         </is>
       </c>
       <c r="AB92" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AC92" s="4" t="inlineStr">
         <is>
@@ -5985,7 +5985,7 @@
         <v>11614</v>
       </c>
       <c r="X93" s="7" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="Y93" s="7" t="inlineStr">
         <is>
@@ -6026,7 +6026,7 @@
         <v>11098</v>
       </c>
       <c r="X94" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y94" s="4" t="inlineStr">
         <is>
@@ -6067,7 +6067,7 @@
         <v>11097</v>
       </c>
       <c r="X95" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y95" s="7" t="inlineStr">
         <is>
@@ -6149,7 +6149,7 @@
         <v>11482</v>
       </c>
       <c r="X97" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Y97" s="7" t="inlineStr">
         <is>
@@ -6231,7 +6231,7 @@
         <v>11380</v>
       </c>
       <c r="X99" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Y99" s="7" t="inlineStr">
         <is>
@@ -6354,7 +6354,7 @@
         <v>11075</v>
       </c>
       <c r="X102" s="4" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="Y102" s="4" t="inlineStr">
         <is>
@@ -6395,7 +6395,7 @@
         <v>11539</v>
       </c>
       <c r="X103" s="7" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="Y103" s="7" t="inlineStr">
         <is>
@@ -6436,7 +6436,7 @@
         <v>11799</v>
       </c>
       <c r="X104" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="Y104" s="4" t="inlineStr">
         <is>
@@ -6477,7 +6477,7 @@
         <v>26509</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="Y105" s="7" t="inlineStr">
         <is>
@@ -6518,20 +6518,20 @@
         <v>26876</v>
       </c>
       <c r="X106" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="Y106" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="Z106" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.pedidosya</t>
+        </is>
+      </c>
+      <c r="AB106" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="Y106" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="Z106" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.pedidosya</t>
-        </is>
-      </c>
-      <c r="AB106" s="4" t="n">
-        <v>22</v>
       </c>
       <c r="AC106" s="4" t="inlineStr">
         <is>
@@ -6559,7 +6559,7 @@
         <v>27154</v>
       </c>
       <c r="X107" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Y107" s="7" t="inlineStr">
         <is>
@@ -6572,7 +6572,7 @@
         </is>
       </c>
       <c r="AB107" s="7" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="AC107" s="7" t="inlineStr">
         <is>
@@ -6600,7 +6600,7 @@
         <v>26655</v>
       </c>
       <c r="X108" s="4" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="Y108" s="4" t="inlineStr">
         <is>
@@ -6613,7 +6613,7 @@
         </is>
       </c>
       <c r="AB108" s="4" t="n">
-        <v>5</v>
+        <v>154</v>
       </c>
       <c r="AC108" s="4" t="inlineStr">
         <is>
@@ -6641,7 +6641,7 @@
         <v>25267</v>
       </c>
       <c r="X109" s="7" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="Y109" s="7" t="inlineStr">
         <is>
@@ -6654,7 +6654,7 @@
         </is>
       </c>
       <c r="AB109" s="7" t="n">
-        <v>154</v>
+        <v>5</v>
       </c>
       <c r="AC109" s="7" t="inlineStr">
         <is>
@@ -6682,7 +6682,7 @@
         <v>24712</v>
       </c>
       <c r="X110" s="4" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="Y110" s="4" t="inlineStr">
         <is>
@@ -6736,7 +6736,7 @@
         </is>
       </c>
       <c r="AB111" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AC111" s="7" t="inlineStr">
         <is>
@@ -6764,7 +6764,7 @@
         <v>25640</v>
       </c>
       <c r="X112" s="4" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="Y112" s="4" t="inlineStr">
         <is>
@@ -6777,7 +6777,7 @@
         </is>
       </c>
       <c r="AB112" s="4" t="n">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="AC112" s="4" t="inlineStr">
         <is>
@@ -6805,7 +6805,7 @@
         <v>26277</v>
       </c>
       <c r="X113" s="7" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="Y113" s="7" t="inlineStr">
         <is>
@@ -6818,7 +6818,7 @@
         </is>
       </c>
       <c r="AB113" s="7" t="n">
-        <v>55</v>
+        <v>4</v>
       </c>
       <c r="AC113" s="7" t="inlineStr">
         <is>
@@ -6846,7 +6846,7 @@
         <v>27017</v>
       </c>
       <c r="X114" s="4" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="Y114" s="4" t="inlineStr">
         <is>
@@ -6859,7 +6859,7 @@
         </is>
       </c>
       <c r="AB114" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC114" s="4" t="inlineStr">
         <is>
@@ -6887,7 +6887,7 @@
         <v>26315</v>
       </c>
       <c r="X115" s="7" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="Y115" s="7" t="inlineStr">
         <is>
@@ -6900,7 +6900,7 @@
         </is>
       </c>
       <c r="AB115" s="7" t="n">
-        <v>3</v>
+        <v>44</v>
       </c>
       <c r="AC115" s="7" t="inlineStr">
         <is>
@@ -6941,7 +6941,7 @@
         </is>
       </c>
       <c r="AB116" s="4" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="AC116" s="4" t="inlineStr">
         <is>
@@ -7297,7 +7297,7 @@
         <v>17825</v>
       </c>
       <c r="X125" s="7" t="n">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="Y125" s="7" t="inlineStr">
         <is>
@@ -7338,7 +7338,7 @@
         <v>17897</v>
       </c>
       <c r="X126" s="4" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="Y126" s="4" t="inlineStr">
         <is>
@@ -7351,7 +7351,7 @@
         </is>
       </c>
       <c r="AB126" s="4" t="n">
-        <v>302</v>
+        <v>4</v>
       </c>
       <c r="AC126" s="4" t="inlineStr">
         <is>
@@ -7392,7 +7392,7 @@
         </is>
       </c>
       <c r="AB127" s="7" t="n">
-        <v>4</v>
+        <v>302</v>
       </c>
       <c r="AC127" s="7" t="inlineStr">
         <is>
@@ -7420,7 +7420,7 @@
         <v>17704</v>
       </c>
       <c r="X128" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Y128" s="4" t="inlineStr">
         <is>
@@ -7433,7 +7433,7 @@
         </is>
       </c>
       <c r="AB128" s="4" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="AC128" s="4" t="inlineStr">
         <is>
@@ -7461,7 +7461,7 @@
         <v>17380</v>
       </c>
       <c r="X129" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Y129" s="7" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         </is>
       </c>
       <c r="AB129" s="7" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="AC129" s="7" t="inlineStr">
         <is>
@@ -7502,7 +7502,7 @@
         <v>17336</v>
       </c>
       <c r="X130" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y130" s="4" t="inlineStr">
         <is>
@@ -7543,7 +7543,7 @@
         <v>17584</v>
       </c>
       <c r="X131" s="7" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="Y131" s="7" t="inlineStr">
         <is>
@@ -7556,7 +7556,7 @@
         </is>
       </c>
       <c r="AB131" s="7" t="n">
-        <v>1</v>
+        <v>158</v>
       </c>
       <c r="AC131" s="7" t="inlineStr">
         <is>
@@ -7584,7 +7584,7 @@
         <v>17915</v>
       </c>
       <c r="X132" s="4" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="Y132" s="4" t="inlineStr">
         <is>
@@ -7597,7 +7597,7 @@
         </is>
       </c>
       <c r="AB132" s="4" t="n">
-        <v>158</v>
+        <v>1</v>
       </c>
       <c r="AC132" s="4" t="inlineStr">
         <is>
@@ -7638,7 +7638,7 @@
         </is>
       </c>
       <c r="AB133" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AC133" s="7" t="inlineStr">
         <is>
@@ -7679,7 +7679,7 @@
         </is>
       </c>
       <c r="AB134" s="4" t="n">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="AC134" s="4" t="inlineStr">
         <is>
@@ -7720,7 +7720,7 @@
         </is>
       </c>
       <c r="AB135" s="7" t="n">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="AC135" s="7" t="inlineStr">
         <is>
@@ -7748,7 +7748,7 @@
         <v>783</v>
       </c>
       <c r="X136" s="4" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="Y136" s="4" t="inlineStr">
         <is>
@@ -7761,7 +7761,7 @@
         </is>
       </c>
       <c r="AB136" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AC136" s="4" t="inlineStr">
         <is>
@@ -7789,7 +7789,7 @@
         <v>763</v>
       </c>
       <c r="X137" s="7" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="Y137" s="7" t="inlineStr">
         <is>
@@ -7802,7 +7802,7 @@
         </is>
       </c>
       <c r="AB137" s="7" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="AC137" s="7" t="inlineStr">
         <is>
@@ -7830,7 +7830,7 @@
         <v>735</v>
       </c>
       <c r="X138" s="4" t="n">
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="Y138" s="4" t="inlineStr">
         <is>
@@ -7843,7 +7843,7 @@
         </is>
       </c>
       <c r="AB138" s="4" t="n">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="AC138" s="4" t="inlineStr">
         <is>
@@ -7871,7 +7871,7 @@
         <v>841</v>
       </c>
       <c r="X139" s="7" t="n">
-        <v>55</v>
+        <v>4</v>
       </c>
       <c r="Y139" s="7" t="inlineStr">
         <is>
@@ -7912,7 +7912,7 @@
         <v>767</v>
       </c>
       <c r="X140" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y140" s="4" t="inlineStr">
         <is>
@@ -7953,7 +7953,7 @@
         <v>748</v>
       </c>
       <c r="X141" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y141" s="7" t="inlineStr">
         <is>
@@ -8035,7 +8035,7 @@
         <v>772</v>
       </c>
       <c r="X143" s="7" t="n">
-        <v>7</v>
+        <v>49</v>
       </c>
       <c r="Y143" s="7" t="inlineStr">
         <is>
@@ -8076,7 +8076,7 @@
         <v>728</v>
       </c>
       <c r="X144" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Y144" s="4" t="inlineStr">
         <is>
@@ -8117,7 +8117,7 @@
         <v>744</v>
       </c>
       <c r="X145" s="7" t="n">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="Y145" s="7" t="inlineStr">
         <is>
@@ -8130,7 +8130,7 @@
         </is>
       </c>
       <c r="AB145" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AC145" s="7" t="inlineStr">
         <is>
@@ -8171,7 +8171,7 @@
         </is>
       </c>
       <c r="AB146" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="AC146" s="4" t="inlineStr">
         <is>
@@ -8253,7 +8253,7 @@
         </is>
       </c>
       <c r="AB148" s="4" t="n">
-        <v>35</v>
+        <v>300</v>
       </c>
       <c r="AC148" s="4" t="inlineStr">
         <is>
@@ -8281,7 +8281,7 @@
         <v>2141</v>
       </c>
       <c r="X149" s="7" t="n">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="Y149" s="7" t="inlineStr">
         <is>
@@ -8322,7 +8322,7 @@
         <v>2082</v>
       </c>
       <c r="X150" s="4" t="n">
-        <v>3</v>
+        <v>58</v>
       </c>
       <c r="Y150" s="4" t="inlineStr">
         <is>
@@ -8335,7 +8335,7 @@
         </is>
       </c>
       <c r="AB150" s="4" t="n">
-        <v>300</v>
+        <v>35</v>
       </c>
       <c r="AC150" s="4" t="inlineStr">
         <is>
@@ -8363,7 +8363,7 @@
         <v>1990</v>
       </c>
       <c r="X151" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Y151" s="7" t="inlineStr">
         <is>
@@ -8376,7 +8376,7 @@
         </is>
       </c>
       <c r="AB151" s="7" t="n">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="AC151" s="7" t="inlineStr">
         <is>
@@ -8404,7 +8404,7 @@
         <v>2043</v>
       </c>
       <c r="X152" s="4" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="Y152" s="4" t="inlineStr">
         <is>
@@ -8417,7 +8417,7 @@
         </is>
       </c>
       <c r="AB152" s="4" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="AC152" s="4" t="inlineStr">
         <is>
@@ -8445,20 +8445,20 @@
         <v>2148</v>
       </c>
       <c r="X153" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="Y153" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="Z153" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="AB153" s="7" t="n">
         <v>5</v>
-      </c>
-      <c r="Y153" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="Z153" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.glovo</t>
-        </is>
-      </c>
-      <c r="AB153" s="7" t="n">
-        <v>139</v>
       </c>
       <c r="AC153" s="7" t="inlineStr">
         <is>
@@ -8486,7 +8486,7 @@
         <v>2096</v>
       </c>
       <c r="X154" s="4" t="n">
-        <v>61</v>
+        <v>6</v>
       </c>
       <c r="Y154" s="4" t="inlineStr">
         <is>
@@ -8499,7 +8499,7 @@
         </is>
       </c>
       <c r="AB154" s="4" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="AC154" s="4" t="inlineStr">
         <is>
@@ -8540,7 +8540,7 @@
         </is>
       </c>
       <c r="AB155" s="7" t="n">
-        <v>15</v>
+        <v>139</v>
       </c>
       <c r="AC155" s="7" t="inlineStr">
         <is>
@@ -8568,7 +8568,7 @@
         <v>2187</v>
       </c>
       <c r="X156" s="4" t="n">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="Y156" s="4" t="inlineStr">
         <is>
@@ -8609,7 +8609,7 @@
         <v>2127</v>
       </c>
       <c r="X157" s="7" t="n">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="Y157" s="7" t="inlineStr">
         <is>
@@ -8650,7 +8650,7 @@
         <v>2022</v>
       </c>
       <c r="X158" s="4" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="Y158" s="4" t="inlineStr">
         <is>
@@ -8691,7 +8691,7 @@
         <v>2040</v>
       </c>
       <c r="X159" s="7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="Y159" s="7" t="inlineStr">
         <is>
@@ -8732,7 +8732,7 @@
         <v>2157</v>
       </c>
       <c r="X160" s="4" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="Y160" s="4" t="inlineStr">
         <is>
@@ -8763,7 +8763,7 @@
       <c r="U161" s="7" t="n"/>
       <c r="V161" s="7" t="n"/>
       <c r="X161" s="7" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="Y161" s="7" t="inlineStr">
         <is>
@@ -8794,7 +8794,7 @@
       <c r="U162" s="4" t="n"/>
       <c r="V162" s="4" t="n"/>
       <c r="X162" s="4" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="Y162" s="4" t="inlineStr">
         <is>
@@ -8825,7 +8825,7 @@
       <c r="U163" s="7" t="n"/>
       <c r="V163" s="7" t="n"/>
       <c r="X163" s="7" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="Y163" s="7" t="inlineStr">
         <is>
@@ -8887,7 +8887,7 @@
       <c r="U165" s="7" t="n"/>
       <c r="V165" s="7" t="n"/>
       <c r="X165" s="7" t="n">
-        <v>2</v>
+        <v>35</v>
       </c>
       <c r="Y165" s="7" t="inlineStr">
         <is>
@@ -8993,7 +8993,7 @@
         </is>
       </c>
       <c r="AB168" s="4" t="n">
-        <v>2</v>
+        <v>291</v>
       </c>
       <c r="AC168" s="4" t="inlineStr">
         <is>
@@ -9011,7 +9011,7 @@
       <c r="U169" s="7" t="n"/>
       <c r="V169" s="7" t="n"/>
       <c r="X169" s="7" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="Y169" s="7" t="inlineStr">
         <is>
@@ -9042,7 +9042,7 @@
       <c r="U170" s="4" t="n"/>
       <c r="V170" s="4" t="n"/>
       <c r="X170" s="4" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="Y170" s="4" t="inlineStr">
         <is>
@@ -9055,7 +9055,7 @@
         </is>
       </c>
       <c r="AB170" s="4" t="n">
-        <v>291</v>
+        <v>2</v>
       </c>
       <c r="AC170" s="4" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
       <c r="U171" s="7" t="n"/>
       <c r="V171" s="7" t="n"/>
       <c r="X171" s="7" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="Y171" s="7" t="inlineStr">
         <is>
@@ -9086,7 +9086,7 @@
         </is>
       </c>
       <c r="AB171" s="7" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="AC171" s="7" t="inlineStr">
         <is>
@@ -9117,7 +9117,7 @@
         </is>
       </c>
       <c r="AB172" s="4" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="AC172" s="4" t="inlineStr">
         <is>
@@ -9148,7 +9148,7 @@
         </is>
       </c>
       <c r="AB173" s="7" t="n">
-        <v>32</v>
+        <v>131</v>
       </c>
       <c r="AC173" s="7" t="inlineStr">
         <is>
@@ -9179,7 +9179,7 @@
         </is>
       </c>
       <c r="AB174" s="4" t="n">
-        <v>131</v>
+        <v>32</v>
       </c>
       <c r="AC174" s="4" t="inlineStr">
         <is>
@@ -9228,7 +9228,7 @@
       <c r="U176" s="4" t="n"/>
       <c r="V176" s="4" t="n"/>
       <c r="X176" s="4" t="n">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="Y176" s="4" t="inlineStr">
         <is>
@@ -9259,7 +9259,7 @@
       <c r="U177" s="7" t="n"/>
       <c r="V177" s="7" t="n"/>
       <c r="X177" s="7" t="n">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="Y177" s="7" t="inlineStr">
         <is>
@@ -9272,7 +9272,7 @@
         </is>
       </c>
       <c r="AB177" s="7" t="n">
-        <v>2</v>
+        <v>63</v>
       </c>
       <c r="AC177" s="7" t="inlineStr">
         <is>
@@ -9303,7 +9303,7 @@
         </is>
       </c>
       <c r="AB178" s="4" t="n">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="AC178" s="4" t="inlineStr">
         <is>
@@ -9365,7 +9365,7 @@
         </is>
       </c>
       <c r="AB180" s="4" t="n">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="AC180" s="4" t="inlineStr">
         <is>
@@ -9458,7 +9458,7 @@
         </is>
       </c>
       <c r="AB183" s="7" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="AC183" s="7" t="inlineStr">
         <is>
@@ -9724,7 +9724,7 @@
       <c r="U192" s="4" t="n"/>
       <c r="V192" s="4" t="n"/>
       <c r="X192" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y192" s="4" t="inlineStr">
         <is>
@@ -9755,7 +9755,7 @@
       <c r="U193" s="7" t="n"/>
       <c r="V193" s="7" t="n"/>
       <c r="X193" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y193" s="7" t="inlineStr">
         <is>
@@ -9786,7 +9786,7 @@
       <c r="U194" s="4" t="n"/>
       <c r="V194" s="4" t="n"/>
       <c r="X194" s="4" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="Y194" s="4" t="inlineStr">
         <is>
@@ -9817,7 +9817,7 @@
       <c r="U195" s="7" t="n"/>
       <c r="V195" s="7" t="n"/>
       <c r="X195" s="7" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="Y195" s="7" t="inlineStr">
         <is>
@@ -9861,7 +9861,7 @@
         </is>
       </c>
       <c r="AB196" s="4" t="n">
-        <v>43</v>
+        <v>132</v>
       </c>
       <c r="AC196" s="4" t="inlineStr">
         <is>
@@ -9892,7 +9892,7 @@
         </is>
       </c>
       <c r="AB197" s="7" t="n">
-        <v>132</v>
+        <v>43</v>
       </c>
       <c r="AC197" s="7" t="inlineStr">
         <is>
@@ -9954,7 +9954,7 @@
         </is>
       </c>
       <c r="AB199" s="7" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="AC199" s="7" t="inlineStr">
         <is>
@@ -9972,7 +9972,7 @@
       <c r="U200" s="4" t="n"/>
       <c r="V200" s="4" t="n"/>
       <c r="X200" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Y200" s="4" t="inlineStr">
         <is>
@@ -10003,7 +10003,7 @@
       <c r="U201" s="7" t="n"/>
       <c r="V201" s="7" t="n"/>
       <c r="X201" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Y201" s="7" t="inlineStr">
         <is>
@@ -10016,7 +10016,7 @@
         </is>
       </c>
       <c r="AB201" s="7" t="n">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="AC201" s="7" t="inlineStr">
         <is>
@@ -10034,7 +10034,7 @@
       <c r="U202" s="4" t="n"/>
       <c r="V202" s="4" t="n"/>
       <c r="X202" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Y202" s="4" t="inlineStr">
         <is>
@@ -10047,7 +10047,7 @@
         </is>
       </c>
       <c r="AB202" s="4" t="n">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="AC202" s="4" t="inlineStr">
         <is>
@@ -10065,7 +10065,7 @@
       <c r="U203" s="7" t="n"/>
       <c r="V203" s="7" t="n"/>
       <c r="X203" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Y203" s="7" t="inlineStr">
         <is>
@@ -10078,7 +10078,7 @@
         </is>
       </c>
       <c r="AB203" s="7" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="AC203" s="7" t="inlineStr">
         <is>
@@ -10140,7 +10140,7 @@
         </is>
       </c>
       <c r="AB205" s="7" t="n">
-        <v>142</v>
+        <v>37</v>
       </c>
       <c r="AC205" s="7" t="inlineStr">
         <is>
@@ -10171,7 +10171,7 @@
         </is>
       </c>
       <c r="AB206" s="4" t="n">
-        <v>37</v>
+        <v>142</v>
       </c>
       <c r="AC206" s="4" t="inlineStr">
         <is>
@@ -10378,7 +10378,7 @@
       <c r="Y213" s="7" t="n"/>
       <c r="Z213" s="7" t="n"/>
       <c r="AB213" s="7" t="n">
-        <v>216</v>
+        <v>87</v>
       </c>
       <c r="AC213" s="7" t="inlineStr">
         <is>
@@ -10420,7 +10420,7 @@
       <c r="Y215" s="7" t="n"/>
       <c r="Z215" s="7" t="n"/>
       <c r="AB215" s="7" t="n">
-        <v>87</v>
+        <v>216</v>
       </c>
       <c r="AC215" s="7" t="inlineStr">
         <is>
@@ -10483,7 +10483,7 @@
       <c r="Y218" s="4" t="n"/>
       <c r="Z218" s="4" t="n"/>
       <c r="AB218" s="4" t="n">
-        <v>90</v>
+        <v>5</v>
       </c>
       <c r="AC218" s="4" t="inlineStr">
         <is>
@@ -10525,7 +10525,7 @@
       <c r="Y220" s="4" t="n"/>
       <c r="Z220" s="4" t="n"/>
       <c r="AB220" s="4" t="n">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="AC220" s="4" t="inlineStr">
         <is>
@@ -10546,7 +10546,7 @@
       <c r="Y221" s="7" t="n"/>
       <c r="Z221" s="7" t="n"/>
       <c r="AB221" s="7" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="AC221" s="7" t="inlineStr">
         <is>
@@ -10567,7 +10567,7 @@
       <c r="Y222" s="4" t="n"/>
       <c r="Z222" s="4" t="n"/>
       <c r="AB222" s="4" t="n">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="AC222" s="4" t="inlineStr">
         <is>
@@ -10609,7 +10609,7 @@
       <c r="Y224" s="4" t="n"/>
       <c r="Z224" s="4" t="n"/>
       <c r="AB224" s="4" t="n">
-        <v>54</v>
+        <v>6</v>
       </c>
       <c r="AC224" s="4" t="inlineStr">
         <is>
@@ -10630,7 +10630,7 @@
       <c r="Y225" s="7" t="n"/>
       <c r="Z225" s="7" t="n"/>
       <c r="AB225" s="7" t="n">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="AC225" s="7" t="inlineStr">
         <is>
@@ -10651,7 +10651,7 @@
       <c r="Y226" s="4" t="n"/>
       <c r="Z226" s="4" t="n"/>
       <c r="AB226" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AC226" s="4" t="inlineStr">
         <is>
@@ -10672,7 +10672,7 @@
       <c r="Y227" s="7" t="n"/>
       <c r="Z227" s="7" t="n"/>
       <c r="AB227" s="7" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="AC227" s="7" t="inlineStr">
         <is>
@@ -10693,7 +10693,7 @@
       <c r="Y228" s="4" t="n"/>
       <c r="Z228" s="4" t="n"/>
       <c r="AB228" s="4" t="n">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="AC228" s="4" t="inlineStr">
         <is>
@@ -10714,7 +10714,7 @@
       <c r="Y229" s="7" t="n"/>
       <c r="Z229" s="7" t="n"/>
       <c r="AB229" s="7" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="AC229" s="7" t="inlineStr">
         <is>
@@ -10819,7 +10819,7 @@
       <c r="Y234" s="4" t="n"/>
       <c r="Z234" s="4" t="n"/>
       <c r="AB234" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AC234" s="4" t="inlineStr">
         <is>
@@ -10840,7 +10840,7 @@
       <c r="Y235" s="7" t="n"/>
       <c r="Z235" s="7" t="n"/>
       <c r="AB235" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AC235" s="7" t="inlineStr">
         <is>
@@ -10945,7 +10945,7 @@
       <c r="Y240" s="4" t="n"/>
       <c r="Z240" s="4" t="n"/>
       <c r="AB240" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AC240" s="4" t="inlineStr">
         <is>
@@ -10966,7 +10966,7 @@
       <c r="Y241" s="7" t="n"/>
       <c r="Z241" s="7" t="n"/>
       <c r="AB241" s="7" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="AC241" s="7" t="inlineStr">
         <is>
@@ -10987,7 +10987,7 @@
       <c r="Y242" s="4" t="n"/>
       <c r="Z242" s="4" t="n"/>
       <c r="AB242" s="4" t="n">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="AC242" s="4" t="inlineStr">
         <is>
@@ -11008,7 +11008,7 @@
       <c r="Y243" s="7" t="n"/>
       <c r="Z243" s="7" t="n"/>
       <c r="AB243" s="7" t="n">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="AC243" s="7" t="inlineStr">
         <is>
@@ -11071,7 +11071,7 @@
       <c r="Y246" s="4" t="n"/>
       <c r="Z246" s="4" t="n"/>
       <c r="AB246" s="4" t="n">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="AC246" s="4" t="inlineStr">
         <is>
@@ -11092,7 +11092,7 @@
       <c r="Y247" s="7" t="n"/>
       <c r="Z247" s="7" t="n"/>
       <c r="AB247" s="7" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="AC247" s="7" t="inlineStr">
         <is>
@@ -11113,7 +11113,7 @@
       <c r="Y248" s="4" t="n"/>
       <c r="Z248" s="4" t="n"/>
       <c r="AB248" s="4" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="AC248" s="4" t="inlineStr">
         <is>
@@ -11134,7 +11134,7 @@
       <c r="Y249" s="7" t="n"/>
       <c r="Z249" s="7" t="n"/>
       <c r="AB249" s="7" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="AC249" s="7" t="inlineStr">
         <is>
@@ -11428,7 +11428,7 @@
       <c r="Y263" s="7" t="n"/>
       <c r="Z263" s="7" t="n"/>
       <c r="AB263" s="7" t="n">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="AC263" s="7" t="inlineStr">
         <is>
@@ -11449,7 +11449,7 @@
       <c r="Y264" s="4" t="n"/>
       <c r="Z264" s="4" t="n"/>
       <c r="AB264" s="4" t="n">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="AC264" s="4" t="inlineStr">
         <is>
@@ -11470,7 +11470,7 @@
       <c r="Y265" s="7" t="n"/>
       <c r="Z265" s="7" t="n"/>
       <c r="AB265" s="7" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="AC265" s="7" t="inlineStr">
         <is>
@@ -11512,7 +11512,7 @@
       <c r="Y267" s="7" t="n"/>
       <c r="Z267" s="7" t="n"/>
       <c r="AB267" s="7" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="AC267" s="7" t="inlineStr">
         <is>
@@ -11743,7 +11743,7 @@
       <c r="Y278" s="4" t="n"/>
       <c r="Z278" s="4" t="n"/>
       <c r="AB278" s="4" t="n">
-        <v>134</v>
+        <v>228</v>
       </c>
       <c r="AC278" s="4" t="inlineStr">
         <is>
@@ -11764,7 +11764,7 @@
       <c r="Y279" s="7" t="n"/>
       <c r="Z279" s="7" t="n"/>
       <c r="AB279" s="7" t="n">
-        <v>228</v>
+        <v>134</v>
       </c>
       <c r="AC279" s="7" t="inlineStr">
         <is>
@@ -11785,7 +11785,7 @@
       <c r="Y280" s="4" t="n"/>
       <c r="Z280" s="4" t="n"/>
       <c r="AB280" s="4" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="AC280" s="4" t="inlineStr">
         <is>
@@ -11806,7 +11806,7 @@
       <c r="Y281" s="7" t="n"/>
       <c r="Z281" s="7" t="n"/>
       <c r="AB281" s="7" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="AC281" s="7" t="inlineStr">
         <is>
@@ -11827,7 +11827,7 @@
       <c r="Y282" s="4" t="n"/>
       <c r="Z282" s="4" t="n"/>
       <c r="AB282" s="4" t="n">
-        <v>60</v>
+        <v>94</v>
       </c>
       <c r="AC282" s="4" t="inlineStr">
         <is>
@@ -11848,7 +11848,7 @@
       <c r="Y283" s="7" t="n"/>
       <c r="Z283" s="7" t="n"/>
       <c r="AB283" s="7" t="n">
-        <v>94</v>
+        <v>60</v>
       </c>
       <c r="AC283" s="7" t="inlineStr">
         <is>
@@ -11890,7 +11890,7 @@
       <c r="Y285" s="7" t="n"/>
       <c r="Z285" s="7" t="n"/>
       <c r="AB285" s="7" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="AC285" s="7" t="inlineStr">
         <is>
@@ -11911,7 +11911,7 @@
       <c r="Y286" s="4" t="n"/>
       <c r="Z286" s="4" t="n"/>
       <c r="AB286" s="4" t="n">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="AC286" s="4" t="inlineStr">
         <is>
@@ -11932,7 +11932,7 @@
       <c r="Y287" s="7" t="n"/>
       <c r="Z287" s="7" t="n"/>
       <c r="AB287" s="7" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="AC287" s="7" t="inlineStr">
         <is>
@@ -11953,7 +11953,7 @@
       <c r="Y288" s="4" t="n"/>
       <c r="Z288" s="4" t="n"/>
       <c r="AB288" s="4" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="AC288" s="4" t="inlineStr">
         <is>
@@ -12079,7 +12079,7 @@
       <c r="Y294" s="4" t="n"/>
       <c r="Z294" s="4" t="n"/>
       <c r="AB294" s="4" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="AC294" s="4" t="inlineStr">
         <is>
@@ -12100,7 +12100,7 @@
       <c r="Y295" s="7" t="n"/>
       <c r="Z295" s="7" t="n"/>
       <c r="AB295" s="7" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="AC295" s="7" t="inlineStr">
         <is>
@@ -12695,7 +12695,7 @@
         </is>
       </c>
       <c r="AB6" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
@@ -12781,7 +12781,7 @@
         </is>
       </c>
       <c r="AB7" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
@@ -13033,7 +13033,7 @@
         </is>
       </c>
       <c r="AB10" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
@@ -13111,7 +13111,7 @@
         </is>
       </c>
       <c r="AB11" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
@@ -13607,7 +13607,7 @@
         </is>
       </c>
       <c r="AB19" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AC19" t="inlineStr">
         <is>
@@ -13653,7 +13653,7 @@
         </is>
       </c>
       <c r="AB20" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="AC20" t="inlineStr">
         <is>
@@ -14358,7 +14358,7 @@
         <v>7963</v>
       </c>
       <c r="X35" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
@@ -14399,20 +14399,20 @@
         <v>11169</v>
       </c>
       <c r="X36" t="n">
+        <v>22</v>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.talabat</t>
+        </is>
+      </c>
+      <c r="AB36" t="n">
         <v>1</v>
-      </c>
-      <c r="Y36" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="Z36" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.talabat</t>
-        </is>
-      </c>
-      <c r="AB36" t="n">
-        <v>3</v>
       </c>
       <c r="AC36" t="inlineStr">
         <is>
@@ -14453,7 +14453,7 @@
         </is>
       </c>
       <c r="AB37" t="n">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="AC37" t="inlineStr">
         <is>
@@ -14494,7 +14494,7 @@
         </is>
       </c>
       <c r="AB38" t="n">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="AC38" t="inlineStr">
         <is>
@@ -14522,7 +14522,7 @@
         <v>11593</v>
       </c>
       <c r="X39" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="Y39" t="inlineStr">
         <is>
@@ -14563,7 +14563,7 @@
         <v>10855</v>
       </c>
       <c r="X40" t="n">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
@@ -14699,7 +14699,7 @@
         </is>
       </c>
       <c r="AB43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC43" t="inlineStr">
         <is>
@@ -14740,7 +14740,7 @@
         </is>
       </c>
       <c r="AB44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC44" t="inlineStr">
         <is>
@@ -14768,7 +14768,7 @@
         <v>3533</v>
       </c>
       <c r="X45" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="Y45" t="inlineStr">
         <is>
@@ -14809,7 +14809,7 @@
         <v>4891</v>
       </c>
       <c r="X46" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="Y46" t="inlineStr">
         <is>
@@ -15068,7 +15068,7 @@
         </is>
       </c>
       <c r="AB52" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AC52" t="inlineStr">
         <is>
@@ -15096,7 +15096,7 @@
         <v>20742</v>
       </c>
       <c r="X53" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Y53" t="inlineStr">
         <is>
@@ -15109,7 +15109,7 @@
         </is>
       </c>
       <c r="AB53" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="AC53" t="inlineStr">
         <is>
@@ -15137,7 +15137,7 @@
         <v>19079</v>
       </c>
       <c r="X54" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Y54" t="inlineStr">
         <is>
@@ -15150,7 +15150,7 @@
         </is>
       </c>
       <c r="AB54" t="n">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="AC54" t="inlineStr">
         <is>
@@ -15191,7 +15191,7 @@
         </is>
       </c>
       <c r="AB55" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="AC55" t="inlineStr">
         <is>
@@ -15314,7 +15314,7 @@
         </is>
       </c>
       <c r="AB58" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="AC58" t="inlineStr">
         <is>
@@ -15355,7 +15355,7 @@
         </is>
       </c>
       <c r="AB59" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="AC59" t="inlineStr">
         <is>
@@ -15383,7 +15383,7 @@
         <v>2882</v>
       </c>
       <c r="X60" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Y60" t="inlineStr">
         <is>
@@ -15396,7 +15396,7 @@
         </is>
       </c>
       <c r="AB60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC60" t="inlineStr">
         <is>
@@ -15424,7 +15424,7 @@
         <v>3280</v>
       </c>
       <c r="X61" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Y61" t="inlineStr">
         <is>
@@ -15465,7 +15465,7 @@
         <v>3951</v>
       </c>
       <c r="X62" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="Y62" t="inlineStr">
         <is>
@@ -15506,7 +15506,7 @@
         <v>5096</v>
       </c>
       <c r="X63" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="Y63" t="inlineStr">
         <is>
@@ -15670,7 +15670,7 @@
         <v>5937</v>
       </c>
       <c r="X67" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Y67" t="inlineStr">
         <is>
@@ -15711,7 +15711,7 @@
         <v>5525</v>
       </c>
       <c r="X68" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Y68" t="inlineStr">
         <is>
@@ -15847,7 +15847,7 @@
         </is>
       </c>
       <c r="AB71" t="n">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="AC71" t="inlineStr">
         <is>
@@ -15888,7 +15888,7 @@
         </is>
       </c>
       <c r="AB72" t="n">
-        <v>3</v>
+        <v>58</v>
       </c>
       <c r="AC72" t="inlineStr">
         <is>
@@ -16052,7 +16052,7 @@
         </is>
       </c>
       <c r="AB76" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="AC76" t="inlineStr">
         <is>
@@ -16093,7 +16093,7 @@
         </is>
       </c>
       <c r="AB77" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="AC77" t="inlineStr">
         <is>
@@ -16134,7 +16134,7 @@
         </is>
       </c>
       <c r="AB78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AC78" t="inlineStr">
         <is>
@@ -16367,7 +16367,7 @@
         <v>975</v>
       </c>
       <c r="X84" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="Y84" t="inlineStr">
         <is>
@@ -16408,7 +16408,7 @@
         <v>622</v>
       </c>
       <c r="X85" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="Y85" t="inlineStr">
         <is>
@@ -16421,7 +16421,7 @@
         </is>
       </c>
       <c r="AB85" t="n">
-        <v>179</v>
+        <v>8</v>
       </c>
       <c r="AC85" t="inlineStr">
         <is>
@@ -16462,7 +16462,7 @@
         </is>
       </c>
       <c r="AB86" t="n">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="AC86" t="inlineStr">
         <is>
@@ -16503,7 +16503,7 @@
         </is>
       </c>
       <c r="AB87" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC87" t="inlineStr">
         <is>
@@ -16544,7 +16544,7 @@
         </is>
       </c>
       <c r="AB88" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="AC88" t="inlineStr">
         <is>
@@ -16572,7 +16572,7 @@
         <v>13894</v>
       </c>
       <c r="X89" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="Y89" t="inlineStr">
         <is>
@@ -16585,7 +16585,7 @@
         </is>
       </c>
       <c r="AB89" t="n">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="AC89" t="inlineStr">
         <is>
@@ -16613,7 +16613,7 @@
         <v>17235</v>
       </c>
       <c r="X90" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="Y90" t="inlineStr">
         <is>
@@ -16654,7 +16654,7 @@
         <v>23145</v>
       </c>
       <c r="X91" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="Y91" t="inlineStr">
         <is>
@@ -16667,7 +16667,7 @@
         </is>
       </c>
       <c r="AB91" t="n">
-        <v>2</v>
+        <v>90</v>
       </c>
       <c r="AC91" t="inlineStr">
         <is>
@@ -16695,7 +16695,7 @@
         <v>32675</v>
       </c>
       <c r="X92" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="Y92" t="inlineStr">
         <is>
@@ -16818,7 +16818,7 @@
         <v>33649</v>
       </c>
       <c r="X95" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="Y95" t="inlineStr">
         <is>
@@ -16859,7 +16859,7 @@
         <v>30739</v>
       </c>
       <c r="X96" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="Y96" t="inlineStr">
         <is>
@@ -16900,7 +16900,7 @@
         <v>27294</v>
       </c>
       <c r="X97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y97" t="inlineStr">
         <is>
@@ -16941,7 +16941,7 @@
         <v>21596</v>
       </c>
       <c r="X98" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="Y98" t="inlineStr">
         <is>
@@ -16982,7 +16982,7 @@
         <v>13483</v>
       </c>
       <c r="X99" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="Y99" t="inlineStr">
         <is>
@@ -17118,7 +17118,7 @@
         </is>
       </c>
       <c r="AB102" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="AC102" t="inlineStr">
         <is>
@@ -17159,7 +17159,7 @@
         </is>
       </c>
       <c r="AB103" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="AC103" t="inlineStr">
         <is>
@@ -17269,7 +17269,7 @@
         <v>354</v>
       </c>
       <c r="X106" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="Y106" t="inlineStr">
         <is>
@@ -17310,7 +17310,7 @@
         <v>347</v>
       </c>
       <c r="X107" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="Y107" t="inlineStr">
         <is>
@@ -17556,7 +17556,7 @@
         <v>176</v>
       </c>
       <c r="X113" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="Y113" t="inlineStr">
         <is>
@@ -17597,7 +17597,7 @@
         <v>603</v>
       </c>
       <c r="X114" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="Y114" t="inlineStr">
         <is>
@@ -18020,7 +18020,7 @@
         </is>
       </c>
       <c r="AB124" t="n">
-        <v>99</v>
+        <v>3</v>
       </c>
       <c r="AC124" t="inlineStr">
         <is>
@@ -18061,7 +18061,7 @@
         </is>
       </c>
       <c r="AB125" t="n">
-        <v>3</v>
+        <v>99</v>
       </c>
       <c r="AC125" t="inlineStr">
         <is>
@@ -18553,7 +18553,7 @@
         </is>
       </c>
       <c r="AB137" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AC137" t="inlineStr">
         <is>
@@ -18609,7 +18609,7 @@
         <v>304</v>
       </c>
       <c r="AB139" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC139" t="inlineStr">
         <is>
@@ -18680,7 +18680,7 @@
     </row>
     <row r="142">
       <c r="AB142" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="AC142" t="inlineStr">
         <is>
@@ -18695,7 +18695,7 @@
     </row>
     <row r="143">
       <c r="AB143" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="AC143" t="inlineStr">
         <is>
@@ -18965,7 +18965,7 @@
     </row>
     <row r="161">
       <c r="AB161" t="n">
-        <v>170</v>
+        <v>1</v>
       </c>
       <c r="AC161" t="inlineStr">
         <is>
@@ -18980,7 +18980,7 @@
     </row>
     <row r="162">
       <c r="AB162" t="n">
-        <v>1</v>
+        <v>170</v>
       </c>
       <c r="AC162" t="inlineStr">
         <is>
@@ -19025,7 +19025,7 @@
     </row>
     <row r="165">
       <c r="AB165" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="AC165" t="inlineStr">
         <is>
@@ -19040,7 +19040,7 @@
     </row>
     <row r="166">
       <c r="AB166" t="n">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="AC166" t="inlineStr">
         <is>
@@ -19100,7 +19100,7 @@
     </row>
     <row r="170">
       <c r="AB170" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="AC170" t="inlineStr">
         <is>
@@ -19115,7 +19115,7 @@
     </row>
     <row r="171">
       <c r="AB171" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="AC171" t="inlineStr">
         <is>
@@ -19235,7 +19235,7 @@
     </row>
     <row r="179">
       <c r="AB179" t="n">
-        <v>3</v>
+        <v>70</v>
       </c>
       <c r="AC179" t="inlineStr">
         <is>
@@ -19250,7 +19250,7 @@
     </row>
     <row r="180">
       <c r="AB180" t="n">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="AC180" t="inlineStr">
         <is>
@@ -19550,7 +19550,7 @@
     </row>
     <row r="200">
       <c r="AB200" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="AC200" t="inlineStr">
         <is>
@@ -19565,7 +19565,7 @@
     </row>
     <row r="201">
       <c r="AB201" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="AC201" t="inlineStr">
         <is>
@@ -19772,7 +19772,7 @@
         <v>4.2</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>0.58</v>
@@ -19808,7 +19808,7 @@
         <v>4.2</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="G3" s="7" t="n">
         <v>0.58</v>
@@ -19844,7 +19844,7 @@
         <v>4.2</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>0.58</v>
@@ -19880,7 +19880,7 @@
         <v>4.2</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>0.58</v>
@@ -19916,7 +19916,7 @@
         <v>4.2</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0.58</v>
@@ -19952,7 +19952,7 @@
         <v>4.2</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>0.58</v>
@@ -19988,7 +19988,7 @@
         <v>4.2</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0.58</v>
@@ -20024,7 +20024,7 @@
         <v>4.2</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>0.58</v>
@@ -20060,7 +20060,7 @@
         <v>4.2</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>0.58</v>
@@ -20096,7 +20096,7 @@
         <v>4.2</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1.12</v>
+        <v>1.13</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>0.58</v>
@@ -23986,7 +23986,7 @@
         <v>4.2</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>0.58</v>
@@ -24022,7 +24022,7 @@
         <v>4.2</v>
       </c>
       <c r="F3" s="7" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="G3" s="7" t="n">
         <v>0.58</v>
@@ -24058,7 +24058,7 @@
         <v>4.2</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>0.58</v>
@@ -24094,7 +24094,7 @@
         <v>4.2</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>0.58</v>
@@ -24130,7 +24130,7 @@
         <v>4.2</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>0.58</v>
@@ -24166,7 +24166,7 @@
         <v>4.2</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>0.58</v>
@@ -24202,7 +24202,7 @@
         <v>4.2</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>0.58</v>
@@ -24238,7 +24238,7 @@
         <v>4.2</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>0.58</v>
@@ -24274,7 +24274,7 @@
         <v>4.2</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>0.58</v>
@@ -24310,7 +24310,7 @@
         <v>4.2</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>1.01</v>
+        <v>1.05</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>0.58</v>

</xml_diff>

<commit_message>
Updated the report to exclude injected hangs from projected report
</commit_message>
<xml_diff>
--- a/consolidation_report/sentry_data.xlsx
+++ b/consolidation_report/sentry_data.xlsx
@@ -1390,7 +1390,7 @@
         </is>
       </c>
       <c r="AB2" s="4" t="n">
-        <v>295</v>
+        <v>6</v>
       </c>
       <c r="AC2" s="4" t="inlineStr">
         <is>
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="AB3" s="7" t="n">
-        <v>6</v>
+        <v>295</v>
       </c>
       <c r="AC3" s="7" t="inlineStr">
         <is>
@@ -1796,7 +1796,7 @@
         <v>1</v>
       </c>
       <c r="X7" s="7" t="n">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="Y7" s="7" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
         <v>1</v>
       </c>
       <c r="X8" s="4" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="Y8" s="4" t="inlineStr">
         <is>
@@ -2047,7 +2047,7 @@
         <v>1</v>
       </c>
       <c r="X10" s="4" t="n">
-        <v>73</v>
+        <v>1</v>
       </c>
       <c r="Y10" s="4" t="inlineStr">
         <is>
@@ -2060,7 +2060,7 @@
         </is>
       </c>
       <c r="AB10" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AC10" s="4" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
         <v>1</v>
       </c>
       <c r="X11" s="7" t="n">
-        <v>1</v>
+        <v>73</v>
       </c>
       <c r="Y11" s="7" t="inlineStr">
         <is>
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="AB11" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AC11" s="7" t="inlineStr">
         <is>
@@ -2284,7 +2284,7 @@
         <v>1</v>
       </c>
       <c r="X13" s="7" t="n">
-        <v>8</v>
+        <v>90</v>
       </c>
       <c r="Y13" s="7" t="inlineStr">
         <is>
@@ -2363,7 +2363,7 @@
         <v>1</v>
       </c>
       <c r="X14" s="4" t="n">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="Y14" s="4" t="inlineStr">
         <is>
@@ -2376,7 +2376,7 @@
         </is>
       </c>
       <c r="AB14" s="4" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="AC14" s="4" t="inlineStr">
         <is>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="AB15" s="7" t="n">
-        <v>3</v>
+        <v>188</v>
       </c>
       <c r="AC15" s="7" t="inlineStr">
         <is>
@@ -2534,7 +2534,7 @@
         </is>
       </c>
       <c r="AB16" s="4" t="n">
-        <v>188</v>
+        <v>13</v>
       </c>
       <c r="AC16" s="4" t="inlineStr">
         <is>
@@ -2600,7 +2600,7 @@
         <v>1</v>
       </c>
       <c r="X17" s="7" t="n">
-        <v>77</v>
+        <v>8</v>
       </c>
       <c r="Y17" s="7" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
         <v>1</v>
       </c>
       <c r="X18" s="4" t="n">
-        <v>8</v>
+        <v>77</v>
       </c>
       <c r="Y18" s="4" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
         <v>1</v>
       </c>
       <c r="X19" s="7" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="Y19" s="7" t="inlineStr">
         <is>
@@ -2837,7 +2837,7 @@
         <v>1</v>
       </c>
       <c r="X20" s="4" t="n">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="Y20" s="4" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
         </is>
       </c>
       <c r="AB20" s="4" t="n">
-        <v>327</v>
+        <v>4</v>
       </c>
       <c r="AC20" s="4" t="inlineStr">
         <is>
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="AB21" s="7" t="n">
-        <v>1</v>
+        <v>327</v>
       </c>
       <c r="AC21" s="7" t="inlineStr">
         <is>
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="AB22" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AC22" s="4" t="inlineStr">
         <is>
@@ -3074,7 +3074,7 @@
         <v>1</v>
       </c>
       <c r="X23" s="7" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="Y23" s="7" t="inlineStr">
         <is>
@@ -3153,7 +3153,7 @@
         <v>1</v>
       </c>
       <c r="X24" s="4" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="Y24" s="4" t="inlineStr">
         <is>
@@ -3212,7 +3212,7 @@
         <v>55</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="Y25" s="7" t="inlineStr">
         <is>
@@ -3271,7 +3271,7 @@
         <v>5519</v>
       </c>
       <c r="X26" s="4" t="n">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="Y26" s="4" t="inlineStr">
         <is>
@@ -3507,7 +3507,7 @@
         <v>5196</v>
       </c>
       <c r="X30" s="4" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="Y30" s="4" t="inlineStr">
         <is>
@@ -3566,7 +3566,7 @@
         <v>5203</v>
       </c>
       <c r="X31" s="7" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="Y31" s="7" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
         <v>5472</v>
       </c>
       <c r="X34" s="4" t="n">
-        <v>84</v>
+        <v>13</v>
       </c>
       <c r="Y34" s="4" t="inlineStr">
         <is>
@@ -3761,7 +3761,7 @@
         </is>
       </c>
       <c r="AB34" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AC34" s="4" t="inlineStr">
         <is>
@@ -3789,7 +3789,7 @@
         <v>5687</v>
       </c>
       <c r="X35" s="7" t="n">
-        <v>13</v>
+        <v>84</v>
       </c>
       <c r="Y35" s="7" t="inlineStr">
         <is>
@@ -3802,7 +3802,7 @@
         </is>
       </c>
       <c r="AB35" s="7" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="AC35" s="7" t="inlineStr">
         <is>
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="AB36" s="4" t="n">
-        <v>5</v>
+        <v>180</v>
       </c>
       <c r="AC36" s="4" t="inlineStr">
         <is>
@@ -3884,7 +3884,7 @@
         </is>
       </c>
       <c r="AB37" s="7" t="n">
-        <v>180</v>
+        <v>10</v>
       </c>
       <c r="AC37" s="7" t="inlineStr">
         <is>
@@ -3912,7 +3912,7 @@
         <v>5547</v>
       </c>
       <c r="X38" s="4" t="n">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="Y38" s="4" t="inlineStr">
         <is>
@@ -3953,7 +3953,7 @@
         <v>5822</v>
       </c>
       <c r="X39" s="7" t="n">
-        <v>70</v>
+        <v>18</v>
       </c>
       <c r="Y39" s="7" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         </is>
       </c>
       <c r="AB42" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AC42" s="4" t="inlineStr">
         <is>
@@ -4130,7 +4130,7 @@
         </is>
       </c>
       <c r="AB43" s="7" t="n">
-        <v>2</v>
+        <v>276</v>
       </c>
       <c r="AC43" s="7" t="inlineStr">
         <is>
@@ -4158,7 +4158,7 @@
         <v>5476</v>
       </c>
       <c r="X44" s="4" t="n">
-        <v>19</v>
+        <v>78</v>
       </c>
       <c r="Y44" s="4" t="inlineStr">
         <is>
@@ -4171,7 +4171,7 @@
         </is>
       </c>
       <c r="AB44" s="4" t="n">
-        <v>276</v>
+        <v>7</v>
       </c>
       <c r="AC44" s="4" t="inlineStr">
         <is>
@@ -4199,7 +4199,7 @@
         <v>5446</v>
       </c>
       <c r="X45" s="7" t="n">
-        <v>78</v>
+        <v>19</v>
       </c>
       <c r="Y45" s="7" t="inlineStr">
         <is>
@@ -4499,7 +4499,7 @@
         </is>
       </c>
       <c r="AB52" s="4" t="n">
-        <v>2</v>
+        <v>59</v>
       </c>
       <c r="AC52" s="4" t="inlineStr">
         <is>
@@ -4527,7 +4527,7 @@
         <v>14553</v>
       </c>
       <c r="X53" s="7" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="Y53" s="7" t="inlineStr">
         <is>
@@ -4540,7 +4540,7 @@
         </is>
       </c>
       <c r="AB53" s="7" t="n">
-        <v>59</v>
+        <v>2</v>
       </c>
       <c r="AC53" s="7" t="inlineStr">
         <is>
@@ -4568,7 +4568,7 @@
         <v>14491</v>
       </c>
       <c r="X54" s="4" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="Y54" s="4" t="inlineStr">
         <is>
@@ -4609,7 +4609,7 @@
         <v>15132</v>
       </c>
       <c r="X55" s="7" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="Y55" s="7" t="inlineStr">
         <is>
@@ -4622,7 +4622,7 @@
         </is>
       </c>
       <c r="AB55" s="7" t="n">
-        <v>10</v>
+        <v>198</v>
       </c>
       <c r="AC55" s="7" t="inlineStr">
         <is>
@@ -4650,20 +4650,20 @@
         <v>15616</v>
       </c>
       <c r="X56" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y56" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="Z56" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.foodora</t>
+        </is>
+      </c>
+      <c r="AB56" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="Y56" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="Z56" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.foodora</t>
-        </is>
-      </c>
-      <c r="AB56" s="4" t="n">
-        <v>7</v>
       </c>
       <c r="AC56" s="4" t="inlineStr">
         <is>
@@ -4691,7 +4691,7 @@
         <v>15857</v>
       </c>
       <c r="X57" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Y57" s="7" t="inlineStr">
         <is>
@@ -4704,7 +4704,7 @@
         </is>
       </c>
       <c r="AB57" s="7" t="n">
-        <v>198</v>
+        <v>7</v>
       </c>
       <c r="AC57" s="7" t="inlineStr">
         <is>
@@ -4732,7 +4732,7 @@
         <v>15396</v>
       </c>
       <c r="X58" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Y58" s="4" t="inlineStr">
         <is>
@@ -4827,7 +4827,7 @@
         </is>
       </c>
       <c r="AB60" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AC60" s="4" t="inlineStr">
         <is>
@@ -4855,7 +4855,7 @@
         <v>14680</v>
       </c>
       <c r="X61" s="7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="Y61" s="7" t="inlineStr">
         <is>
@@ -4868,7 +4868,7 @@
         </is>
       </c>
       <c r="AB61" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AC61" s="7" t="inlineStr">
         <is>
@@ -4896,7 +4896,7 @@
         <v>15388</v>
       </c>
       <c r="X62" s="4" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Y62" s="4" t="inlineStr">
         <is>
@@ -5019,7 +5019,7 @@
         <v>15462</v>
       </c>
       <c r="X65" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Y65" s="7" t="inlineStr">
         <is>
@@ -5060,7 +5060,7 @@
         <v>15905</v>
       </c>
       <c r="X66" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Y66" s="4" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
         </is>
       </c>
       <c r="AB66" s="4" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="AC66" s="4" t="inlineStr">
         <is>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="AB67" s="7" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="AC67" s="7" t="inlineStr">
         <is>
@@ -5319,7 +5319,7 @@
         </is>
       </c>
       <c r="AB72" s="4" t="n">
-        <v>7</v>
+        <v>64</v>
       </c>
       <c r="AC72" s="4" t="inlineStr">
         <is>
@@ -5360,7 +5360,7 @@
         </is>
       </c>
       <c r="AB73" s="7" t="n">
-        <v>64</v>
+        <v>7</v>
       </c>
       <c r="AC73" s="7" t="inlineStr">
         <is>
@@ -5401,7 +5401,7 @@
         </is>
       </c>
       <c r="AB74" s="4" t="n">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="AC74" s="4" t="inlineStr">
         <is>
@@ -5429,7 +5429,7 @@
         <v>82796</v>
       </c>
       <c r="X75" s="7" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="Y75" s="7" t="inlineStr">
         <is>
@@ -5442,7 +5442,7 @@
         </is>
       </c>
       <c r="AB75" s="7" t="n">
-        <v>2</v>
+        <v>47</v>
       </c>
       <c r="AC75" s="7" t="inlineStr">
         <is>
@@ -5470,7 +5470,7 @@
         <v>80792</v>
       </c>
       <c r="X76" s="4" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="Y76" s="4" t="inlineStr">
         <is>
@@ -5524,7 +5524,7 @@
         </is>
       </c>
       <c r="AB77" s="7" t="n">
-        <v>157</v>
+        <v>5</v>
       </c>
       <c r="AC77" s="7" t="inlineStr">
         <is>
@@ -5565,7 +5565,7 @@
         </is>
       </c>
       <c r="AB78" s="4" t="n">
-        <v>5</v>
+        <v>157</v>
       </c>
       <c r="AC78" s="4" t="inlineStr">
         <is>
@@ -5729,7 +5729,7 @@
         </is>
       </c>
       <c r="AB82" s="4" t="n">
-        <v>3</v>
+        <v>327</v>
       </c>
       <c r="AC82" s="4" t="inlineStr">
         <is>
@@ -5770,7 +5770,7 @@
         </is>
       </c>
       <c r="AB83" s="7" t="n">
-        <v>327</v>
+        <v>3</v>
       </c>
       <c r="AC83" s="7" t="inlineStr">
         <is>
@@ -5811,7 +5811,7 @@
         </is>
       </c>
       <c r="AB84" s="4" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="AC84" s="4" t="inlineStr">
         <is>
@@ -5852,7 +5852,7 @@
         </is>
       </c>
       <c r="AB85" s="7" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="AC85" s="7" t="inlineStr">
         <is>
@@ -5934,7 +5934,7 @@
         </is>
       </c>
       <c r="AB87" s="7" t="n">
-        <v>157</v>
+        <v>1</v>
       </c>
       <c r="AC87" s="7" t="inlineStr">
         <is>
@@ -5975,7 +5975,7 @@
         </is>
       </c>
       <c r="AB88" s="4" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="AC88" s="4" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
         </is>
       </c>
       <c r="AB90" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AC90" s="4" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
         </is>
       </c>
       <c r="AB91" s="7" t="n">
-        <v>67</v>
+        <v>6</v>
       </c>
       <c r="AC91" s="7" t="inlineStr">
         <is>
@@ -6139,7 +6139,7 @@
         </is>
       </c>
       <c r="AB92" s="4" t="n">
-        <v>4</v>
+        <v>67</v>
       </c>
       <c r="AC92" s="4" t="inlineStr">
         <is>
@@ -6180,7 +6180,7 @@
         </is>
       </c>
       <c r="AB93" s="7" t="n">
-        <v>4</v>
+        <v>44</v>
       </c>
       <c r="AC93" s="7" t="inlineStr">
         <is>
@@ -6221,7 +6221,7 @@
         </is>
       </c>
       <c r="AB94" s="4" t="n">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="AC94" s="4" t="inlineStr">
         <is>
@@ -6262,7 +6262,7 @@
         </is>
       </c>
       <c r="AB95" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AC95" s="7" t="inlineStr">
         <is>
@@ -6303,7 +6303,7 @@
         </is>
       </c>
       <c r="AB96" s="4" t="n">
-        <v>173</v>
+        <v>1</v>
       </c>
       <c r="AC96" s="4" t="inlineStr">
         <is>
@@ -6331,7 +6331,7 @@
         <v>717</v>
       </c>
       <c r="X97" s="7" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="Y97" s="7" t="inlineStr">
         <is>
@@ -6344,7 +6344,7 @@
         </is>
       </c>
       <c r="AB97" s="7" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="AC97" s="7" t="inlineStr">
         <is>
@@ -6372,7 +6372,7 @@
         <v>753</v>
       </c>
       <c r="X98" s="4" t="n">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="Y98" s="4" t="inlineStr">
         <is>
@@ -6385,7 +6385,7 @@
         </is>
       </c>
       <c r="AB98" s="4" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AC98" s="4" t="inlineStr">
         <is>
@@ -6426,7 +6426,7 @@
         </is>
       </c>
       <c r="AB99" s="7" t="n">
-        <v>1</v>
+        <v>173</v>
       </c>
       <c r="AC99" s="7" t="inlineStr">
         <is>
@@ -6495,7 +6495,7 @@
         <v>743</v>
       </c>
       <c r="X101" s="7" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="Y101" s="7" t="inlineStr">
         <is>
@@ -6536,7 +6536,7 @@
         <v>714</v>
       </c>
       <c r="X102" s="4" t="n">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="Y102" s="4" t="inlineStr">
         <is>
@@ -6577,7 +6577,7 @@
         <v>733</v>
       </c>
       <c r="X103" s="7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="Y103" s="7" t="inlineStr">
         <is>
@@ -6618,7 +6618,7 @@
         <v>737</v>
       </c>
       <c r="X104" s="4" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="Y104" s="4" t="inlineStr">
         <is>
@@ -6659,7 +6659,7 @@
         <v>736</v>
       </c>
       <c r="X105" s="7" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="Y105" s="7" t="inlineStr">
         <is>
@@ -6741,7 +6741,7 @@
         <v>701</v>
       </c>
       <c r="X107" s="7" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="Y107" s="7" t="inlineStr">
         <is>
@@ -6782,7 +6782,7 @@
         <v>736</v>
       </c>
       <c r="X108" s="4" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="Y108" s="4" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
         <v>731</v>
       </c>
       <c r="X109" s="7" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="Y109" s="7" t="inlineStr">
         <is>
@@ -6836,7 +6836,7 @@
         </is>
       </c>
       <c r="AB109" s="7" t="n">
-        <v>154</v>
+        <v>3</v>
       </c>
       <c r="AC109" s="7" t="inlineStr">
         <is>
@@ -6877,7 +6877,7 @@
         </is>
       </c>
       <c r="AB110" s="4" t="n">
-        <v>3</v>
+        <v>154</v>
       </c>
       <c r="AC110" s="4" t="inlineStr">
         <is>
@@ -6946,7 +6946,7 @@
         <v>712</v>
       </c>
       <c r="X112" s="4" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="Y112" s="4" t="inlineStr">
         <is>
@@ -6959,7 +6959,7 @@
         </is>
       </c>
       <c r="AB112" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AC112" s="4" t="inlineStr">
         <is>
@@ -7000,7 +7000,7 @@
         </is>
       </c>
       <c r="AB113" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AC113" s="7" t="inlineStr">
         <is>
@@ -7028,7 +7028,7 @@
         <v>701</v>
       </c>
       <c r="X114" s="4" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="Y114" s="4" t="inlineStr">
         <is>
@@ -7164,7 +7164,7 @@
         </is>
       </c>
       <c r="AB117" s="7" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="AC117" s="7" t="inlineStr">
         <is>
@@ -7205,7 +7205,7 @@
         </is>
       </c>
       <c r="AB118" s="4" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="AC118" s="4" t="inlineStr">
         <is>
@@ -7233,7 +7233,7 @@
         <v>51501</v>
       </c>
       <c r="X119" s="7" t="n">
-        <v>7</v>
+        <v>48</v>
       </c>
       <c r="Y119" s="7" t="inlineStr">
         <is>
@@ -7274,7 +7274,7 @@
         <v>51715</v>
       </c>
       <c r="X120" s="4" t="n">
-        <v>48</v>
+        <v>7</v>
       </c>
       <c r="Y120" s="4" t="inlineStr">
         <is>
@@ -7479,7 +7479,7 @@
         <v>50744</v>
       </c>
       <c r="X125" s="7" t="n">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="Y125" s="7" t="inlineStr">
         <is>
@@ -7520,7 +7520,7 @@
         <v>50396</v>
       </c>
       <c r="X126" s="4" t="n">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="Y126" s="4" t="inlineStr">
         <is>
@@ -7561,7 +7561,7 @@
         <v>51782</v>
       </c>
       <c r="X127" s="7" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="Y127" s="7" t="inlineStr">
         <is>
@@ -7602,7 +7602,7 @@
         <v>50710</v>
       </c>
       <c r="X128" s="4" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="Y128" s="4" t="inlineStr">
         <is>
@@ -7615,7 +7615,7 @@
         </is>
       </c>
       <c r="AB128" s="4" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="AC128" s="4" t="inlineStr">
         <is>
@@ -7643,7 +7643,7 @@
         <v>49774</v>
       </c>
       <c r="X129" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y129" s="7" t="inlineStr">
         <is>
@@ -7656,7 +7656,7 @@
         </is>
       </c>
       <c r="AB129" s="7" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="AC129" s="7" t="inlineStr">
         <is>
@@ -7684,7 +7684,7 @@
         <v>49626</v>
       </c>
       <c r="X130" s="4" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="Y130" s="4" t="inlineStr">
         <is>
@@ -7725,7 +7725,7 @@
         <v>51869</v>
       </c>
       <c r="X131" s="7" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="Y131" s="7" t="inlineStr">
         <is>
@@ -7738,7 +7738,7 @@
         </is>
       </c>
       <c r="AB131" s="7" t="n">
-        <v>1</v>
+        <v>158</v>
       </c>
       <c r="AC131" s="7" t="inlineStr">
         <is>
@@ -7779,7 +7779,7 @@
         </is>
       </c>
       <c r="AB132" s="4" t="n">
-        <v>158</v>
+        <v>1</v>
       </c>
       <c r="AC132" s="4" t="inlineStr">
         <is>
@@ -7807,7 +7807,7 @@
         <v>51059</v>
       </c>
       <c r="X133" s="7" t="n">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="Y133" s="7" t="inlineStr">
         <is>
@@ -7820,7 +7820,7 @@
         </is>
       </c>
       <c r="AB133" s="7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AC133" s="7" t="inlineStr">
         <is>
@@ -7861,7 +7861,7 @@
         </is>
       </c>
       <c r="AB134" s="4" t="n">
-        <v>4</v>
+        <v>58</v>
       </c>
       <c r="AC134" s="4" t="inlineStr">
         <is>
@@ -7889,7 +7889,7 @@
         <v>51562</v>
       </c>
       <c r="X135" s="7" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="Y135" s="7" t="inlineStr">
         <is>
@@ -7902,7 +7902,7 @@
         </is>
       </c>
       <c r="AB135" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AC135" s="7" t="inlineStr">
         <is>
@@ -7930,7 +7930,7 @@
         <v>50612</v>
       </c>
       <c r="X136" s="4" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="Y136" s="4" t="inlineStr">
         <is>
@@ -7943,7 +7943,7 @@
         </is>
       </c>
       <c r="AB136" s="4" t="n">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="AC136" s="4" t="inlineStr">
         <is>
@@ -7984,7 +7984,7 @@
         </is>
       </c>
       <c r="AB137" s="7" t="n">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="AC137" s="7" t="inlineStr">
         <is>
@@ -8025,7 +8025,7 @@
         </is>
       </c>
       <c r="AB138" s="4" t="n">
-        <v>43</v>
+        <v>3</v>
       </c>
       <c r="AC138" s="4" t="inlineStr">
         <is>
@@ -8066,7 +8066,7 @@
         </is>
       </c>
       <c r="AB139" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AC139" s="7" t="inlineStr">
         <is>
@@ -8107,7 +8107,7 @@
         </is>
       </c>
       <c r="AB140" s="4" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="AC140" s="4" t="inlineStr">
         <is>
@@ -8148,7 +8148,7 @@
         </is>
       </c>
       <c r="AB141" s="7" t="n">
-        <v>2</v>
+        <v>161</v>
       </c>
       <c r="AC141" s="7" t="inlineStr">
         <is>
@@ -8189,7 +8189,7 @@
         </is>
       </c>
       <c r="AB142" s="4" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="AC142" s="4" t="inlineStr">
         <is>
@@ -8230,7 +8230,7 @@
         </is>
       </c>
       <c r="AB143" s="7" t="n">
-        <v>161</v>
+        <v>2</v>
       </c>
       <c r="AC143" s="7" t="inlineStr">
         <is>
@@ -8258,7 +8258,7 @@
         <v>1</v>
       </c>
       <c r="X144" s="4" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="Y144" s="4" t="inlineStr">
         <is>
@@ -8299,7 +8299,7 @@
         <v>1</v>
       </c>
       <c r="X145" s="7" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="Y145" s="7" t="inlineStr">
         <is>
@@ -8312,7 +8312,7 @@
         </is>
       </c>
       <c r="AB145" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="AC145" s="7" t="inlineStr">
         <is>
@@ -8340,7 +8340,7 @@
         <v>1</v>
       </c>
       <c r="X146" s="4" t="n">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="Y146" s="4" t="inlineStr">
         <is>
@@ -8353,7 +8353,7 @@
         </is>
       </c>
       <c r="AB146" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="AC146" s="4" t="inlineStr">
         <is>
@@ -8381,7 +8381,7 @@
         <v>1</v>
       </c>
       <c r="X147" s="7" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="Y147" s="7" t="inlineStr">
         <is>
@@ -8435,7 +8435,7 @@
         </is>
       </c>
       <c r="AB148" s="4" t="n">
-        <v>1</v>
+        <v>300</v>
       </c>
       <c r="AC148" s="4" t="inlineStr">
         <is>
@@ -8504,7 +8504,7 @@
         <v>1</v>
       </c>
       <c r="X150" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y150" s="4" t="inlineStr">
         <is>
@@ -8517,7 +8517,7 @@
         </is>
       </c>
       <c r="AB150" s="4" t="n">
-        <v>300</v>
+        <v>1</v>
       </c>
       <c r="AC150" s="4" t="inlineStr">
         <is>
@@ -8545,7 +8545,7 @@
         <v>1</v>
       </c>
       <c r="X151" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y151" s="7" t="inlineStr">
         <is>
@@ -8627,7 +8627,7 @@
         <v>1</v>
       </c>
       <c r="X153" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Y153" s="7" t="inlineStr">
         <is>
@@ -8640,7 +8640,7 @@
         </is>
       </c>
       <c r="AB153" s="7" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="AC153" s="7" t="inlineStr">
         <is>
@@ -8668,7 +8668,7 @@
         <v>1</v>
       </c>
       <c r="X154" s="4" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="Y154" s="4" t="inlineStr">
         <is>
@@ -8681,7 +8681,7 @@
         </is>
       </c>
       <c r="AB154" s="4" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="AC154" s="4" t="inlineStr">
         <is>
@@ -8709,7 +8709,7 @@
         <v>1</v>
       </c>
       <c r="X155" s="7" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="Y155" s="7" t="inlineStr">
         <is>
@@ -8750,7 +8750,7 @@
         <v>1</v>
       </c>
       <c r="X156" s="4" t="n">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="Y156" s="4" t="inlineStr">
         <is>
@@ -8791,7 +8791,7 @@
         <v>1</v>
       </c>
       <c r="X157" s="7" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="Y157" s="7" t="inlineStr">
         <is>
@@ -8832,7 +8832,7 @@
         <v>1</v>
       </c>
       <c r="X158" s="4" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="Y158" s="4" t="inlineStr">
         <is>
@@ -8873,7 +8873,7 @@
         <v>11599</v>
       </c>
       <c r="X159" s="7" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="Y159" s="7" t="inlineStr">
         <is>
@@ -8968,7 +8968,7 @@
         </is>
       </c>
       <c r="AB161" s="7" t="n">
-        <v>149</v>
+        <v>1</v>
       </c>
       <c r="AC161" s="7" t="inlineStr">
         <is>
@@ -8996,7 +8996,7 @@
         <v>11098</v>
       </c>
       <c r="X162" s="4" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="Y162" s="4" t="inlineStr">
         <is>
@@ -9037,7 +9037,7 @@
         <v>11097</v>
       </c>
       <c r="X163" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Y163" s="7" t="inlineStr">
         <is>
@@ -9050,7 +9050,7 @@
         </is>
       </c>
       <c r="AB163" s="7" t="n">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="AC163" s="7" t="inlineStr">
         <is>
@@ -9078,7 +9078,7 @@
         <v>11410</v>
       </c>
       <c r="X164" s="4" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="Y164" s="4" t="inlineStr">
         <is>
@@ -9091,7 +9091,7 @@
         </is>
       </c>
       <c r="AB164" s="4" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="AC164" s="4" t="inlineStr">
         <is>
@@ -9119,7 +9119,7 @@
         <v>11482</v>
       </c>
       <c r="X165" s="7" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="Y165" s="7" t="inlineStr">
         <is>
@@ -9132,7 +9132,7 @@
         </is>
       </c>
       <c r="AB165" s="7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AC165" s="7" t="inlineStr">
         <is>
@@ -9160,7 +9160,7 @@
         <v>11322</v>
       </c>
       <c r="X166" s="4" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="Y166" s="4" t="inlineStr">
         <is>
@@ -9173,7 +9173,7 @@
         </is>
       </c>
       <c r="AB166" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="AC166" s="4" t="inlineStr">
         <is>
@@ -9255,7 +9255,7 @@
         </is>
       </c>
       <c r="AB168" s="4" t="n">
-        <v>291</v>
+        <v>55</v>
       </c>
       <c r="AC168" s="4" t="inlineStr">
         <is>
@@ -9296,7 +9296,7 @@
         </is>
       </c>
       <c r="AB169" s="7" t="n">
-        <v>55</v>
+        <v>291</v>
       </c>
       <c r="AC169" s="7" t="inlineStr">
         <is>
@@ -9324,7 +9324,7 @@
         <v>11075</v>
       </c>
       <c r="X170" s="4" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="Y170" s="4" t="inlineStr">
         <is>
@@ -9365,7 +9365,7 @@
         <v>11539</v>
       </c>
       <c r="X171" s="7" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="Y171" s="7" t="inlineStr">
         <is>
@@ -9378,7 +9378,7 @@
         </is>
       </c>
       <c r="AB171" s="7" t="n">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="AC171" s="7" t="inlineStr">
         <is>
@@ -9406,7 +9406,7 @@
         <v>11799</v>
       </c>
       <c r="X172" s="4" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="Y172" s="4" t="inlineStr">
         <is>
@@ -9419,7 +9419,7 @@
         </is>
       </c>
       <c r="AB172" s="4" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="AC172" s="4" t="inlineStr">
         <is>
@@ -9447,7 +9447,7 @@
         <v>11712</v>
       </c>
       <c r="X173" s="7" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="Y173" s="7" t="inlineStr">
         <is>
@@ -9488,7 +9488,7 @@
         <v>11683</v>
       </c>
       <c r="X174" s="4" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="Y174" s="4" t="inlineStr">
         <is>
@@ -9529,7 +9529,7 @@
         <v>11729</v>
       </c>
       <c r="X175" s="7" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="Y175" s="7" t="inlineStr">
         <is>
@@ -9665,7 +9665,7 @@
         </is>
       </c>
       <c r="AB178" s="4" t="n">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="AC178" s="4" t="inlineStr">
         <is>
@@ -9706,7 +9706,7 @@
         </is>
       </c>
       <c r="AB179" s="7" t="n">
-        <v>16</v>
+        <v>63</v>
       </c>
       <c r="AC179" s="7" t="inlineStr">
         <is>
@@ -9747,7 +9747,7 @@
         </is>
       </c>
       <c r="AB180" s="4" t="n">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="AC180" s="4" t="inlineStr">
         <is>
@@ -9788,7 +9788,7 @@
         </is>
       </c>
       <c r="AB181" s="7" t="n">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="AC181" s="7" t="inlineStr">
         <is>
@@ -9870,7 +9870,7 @@
         </is>
       </c>
       <c r="AB183" s="7" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="AC183" s="7" t="inlineStr">
         <is>
@@ -9898,7 +9898,7 @@
         <v>26876</v>
       </c>
       <c r="X184" s="4" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="Y184" s="4" t="inlineStr">
         <is>
@@ -9911,7 +9911,7 @@
         </is>
       </c>
       <c r="AB184" s="4" t="n">
-        <v>137</v>
+        <v>22</v>
       </c>
       <c r="AC184" s="4" t="inlineStr">
         <is>
@@ -9939,7 +9939,7 @@
         <v>27154</v>
       </c>
       <c r="X185" s="7" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="Y185" s="7" t="inlineStr">
         <is>
@@ -9980,7 +9980,7 @@
         <v>26655</v>
       </c>
       <c r="X186" s="4" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="Y186" s="4" t="inlineStr">
         <is>
@@ -9993,7 +9993,7 @@
         </is>
       </c>
       <c r="AB186" s="4" t="n">
-        <v>22</v>
+        <v>137</v>
       </c>
       <c r="AC186" s="4" t="inlineStr">
         <is>
@@ -10021,7 +10021,7 @@
         <v>25267</v>
       </c>
       <c r="X187" s="7" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="Y187" s="7" t="inlineStr">
         <is>
@@ -10116,7 +10116,7 @@
         </is>
       </c>
       <c r="AB189" s="7" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="AC189" s="7" t="inlineStr">
         <is>
@@ -10157,7 +10157,7 @@
         </is>
       </c>
       <c r="AB190" s="4" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="AC190" s="4" t="inlineStr">
         <is>
@@ -10185,7 +10185,7 @@
         <v>26277</v>
       </c>
       <c r="X191" s="7" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="Y191" s="7" t="inlineStr">
         <is>
@@ -10226,7 +10226,7 @@
         <v>27017</v>
       </c>
       <c r="X192" s="4" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="Y192" s="4" t="inlineStr">
         <is>
@@ -10239,7 +10239,7 @@
         </is>
       </c>
       <c r="AB192" s="4" t="n">
-        <v>268</v>
+        <v>72</v>
       </c>
       <c r="AC192" s="4" t="inlineStr">
         <is>
@@ -10280,7 +10280,7 @@
         </is>
       </c>
       <c r="AB193" s="7" t="n">
-        <v>72</v>
+        <v>268</v>
       </c>
       <c r="AC193" s="7" t="inlineStr">
         <is>
@@ -10349,7 +10349,7 @@
         <v>26408</v>
       </c>
       <c r="X195" s="7" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="Y195" s="7" t="inlineStr">
         <is>
@@ -10390,7 +10390,7 @@
         <v>26352</v>
       </c>
       <c r="X196" s="4" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="Y196" s="4" t="inlineStr">
         <is>
@@ -10444,7 +10444,7 @@
         </is>
       </c>
       <c r="AB197" s="7" t="n">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="AC197" s="7" t="inlineStr">
         <is>
@@ -10485,7 +10485,7 @@
         </is>
       </c>
       <c r="AB198" s="4" t="n">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="AC198" s="4" t="inlineStr">
         <is>
@@ -10526,7 +10526,7 @@
         </is>
       </c>
       <c r="AB199" s="7" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="AC199" s="7" t="inlineStr">
         <is>
@@ -10608,7 +10608,7 @@
         </is>
       </c>
       <c r="AB201" s="7" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="AC201" s="7" t="inlineStr">
         <is>
@@ -10636,7 +10636,7 @@
         <v>24680</v>
       </c>
       <c r="X202" s="4" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="Y202" s="4" t="inlineStr">
         <is>
@@ -10649,7 +10649,7 @@
         </is>
       </c>
       <c r="AB202" s="4" t="n">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="AC202" s="4" t="inlineStr">
         <is>
@@ -10718,7 +10718,7 @@
         <v>25365</v>
       </c>
       <c r="X204" s="4" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="Y204" s="4" t="inlineStr">
         <is>
@@ -10731,7 +10731,7 @@
         </is>
       </c>
       <c r="AB204" s="4" t="n">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="AC204" s="4" t="inlineStr">
         <is>
@@ -10800,7 +10800,7 @@
         <v>17949</v>
       </c>
       <c r="X206" s="4" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="Y206" s="4" t="inlineStr">
         <is>
@@ -10841,7 +10841,7 @@
         <v>17549</v>
       </c>
       <c r="X207" s="7" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="Y207" s="7" t="inlineStr">
         <is>
@@ -10882,7 +10882,7 @@
         <v>17646</v>
       </c>
       <c r="X208" s="4" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="Y208" s="4" t="inlineStr">
         <is>
@@ -10923,7 +10923,7 @@
         <v>17131</v>
       </c>
       <c r="X209" s="7" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="Y209" s="7" t="inlineStr">
         <is>
@@ -10964,20 +10964,20 @@
         <v>17470</v>
       </c>
       <c r="X210" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="Y210" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="Z210" s="4" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.hungerstation</t>
+        </is>
+      </c>
+      <c r="AB210" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="Y210" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="Z210" s="4" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.hungerstation</t>
-        </is>
-      </c>
-      <c r="AB210" s="4" t="n">
-        <v>5</v>
       </c>
       <c r="AC210" s="4" t="inlineStr">
         <is>
@@ -11005,7 +11005,7 @@
         <v>17485</v>
       </c>
       <c r="X211" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Y211" s="7" t="inlineStr">
         <is>
@@ -11018,7 +11018,7 @@
         </is>
       </c>
       <c r="AB211" s="7" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="AC211" s="7" t="inlineStr">
         <is>
@@ -11100,7 +11100,7 @@
         </is>
       </c>
       <c r="AB213" s="7" t="n">
-        <v>216</v>
+        <v>1</v>
       </c>
       <c r="AC213" s="7" t="inlineStr">
         <is>
@@ -11182,7 +11182,7 @@
         </is>
       </c>
       <c r="AB215" s="7" t="n">
-        <v>1</v>
+        <v>216</v>
       </c>
       <c r="AC215" s="7" t="inlineStr">
         <is>
@@ -11374,7 +11374,7 @@
         <v>18111</v>
       </c>
       <c r="X220" s="4" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="Y220" s="4" t="inlineStr">
         <is>
@@ -11415,7 +11415,7 @@
         <v>17792</v>
       </c>
       <c r="X221" s="7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Y221" s="7" t="inlineStr">
         <is>
@@ -11456,7 +11456,7 @@
         <v>17777</v>
       </c>
       <c r="X222" s="4" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="Y222" s="4" t="inlineStr">
         <is>
@@ -11497,7 +11497,7 @@
         <v>17292</v>
       </c>
       <c r="X223" s="7" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="Y223" s="7" t="inlineStr">
         <is>
@@ -11510,7 +11510,7 @@
         </is>
       </c>
       <c r="AB223" s="7" t="n">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="AC223" s="7" t="inlineStr">
         <is>
@@ -11551,7 +11551,7 @@
         </is>
       </c>
       <c r="AB224" s="4" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="AC224" s="4" t="inlineStr">
         <is>
@@ -11633,7 +11633,7 @@
         </is>
       </c>
       <c r="AB226" s="4" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="AC226" s="4" t="inlineStr">
         <is>
@@ -11674,7 +11674,7 @@
         </is>
       </c>
       <c r="AB227" s="7" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="AC227" s="7" t="inlineStr">
         <is>
@@ -11702,7 +11702,7 @@
         <v>17803</v>
       </c>
       <c r="X228" s="4" t="n">
-        <v>4</v>
+        <v>55</v>
       </c>
       <c r="Y228" s="4" t="inlineStr">
         <is>
@@ -11743,7 +11743,7 @@
         <v>745</v>
       </c>
       <c r="X229" s="7" t="n">
-        <v>55</v>
+        <v>4</v>
       </c>
       <c r="Y229" s="7" t="inlineStr">
         <is>
@@ -11756,7 +11756,7 @@
         </is>
       </c>
       <c r="AB229" s="7" t="n">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="AC229" s="7" t="inlineStr">
         <is>
@@ -11784,7 +11784,7 @@
         <v>763</v>
       </c>
       <c r="X230" s="4" t="n">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="Y230" s="4" t="inlineStr">
         <is>
@@ -11825,7 +11825,7 @@
         <v>740</v>
       </c>
       <c r="X231" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y231" s="7" t="inlineStr">
         <is>
@@ -11838,7 +11838,7 @@
         </is>
       </c>
       <c r="AB231" s="7" t="n">
-        <v>124</v>
+        <v>51</v>
       </c>
       <c r="AC231" s="7" t="inlineStr">
         <is>
@@ -11866,7 +11866,7 @@
         <v>783</v>
       </c>
       <c r="X232" s="4" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="Y232" s="4" t="inlineStr">
         <is>
@@ -11879,7 +11879,7 @@
         </is>
       </c>
       <c r="AB232" s="4" t="n">
-        <v>51</v>
+        <v>124</v>
       </c>
       <c r="AC232" s="4" t="inlineStr">
         <is>
@@ -11907,7 +11907,7 @@
         <v>763</v>
       </c>
       <c r="X233" s="7" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="Y233" s="7" t="inlineStr">
         <is>
@@ -11989,7 +11989,7 @@
         <v>841</v>
       </c>
       <c r="X235" s="7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Y235" s="7" t="inlineStr">
         <is>
@@ -12125,7 +12125,7 @@
         </is>
       </c>
       <c r="AB238" s="4" t="n">
-        <v>141</v>
+        <v>248</v>
       </c>
       <c r="AC238" s="4" t="inlineStr">
         <is>
@@ -12153,7 +12153,7 @@
         <v>772</v>
       </c>
       <c r="X239" s="7" t="n">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="Y239" s="7" t="inlineStr">
         <is>
@@ -12166,7 +12166,7 @@
         </is>
       </c>
       <c r="AB239" s="7" t="n">
-        <v>248</v>
+        <v>141</v>
       </c>
       <c r="AC239" s="7" t="inlineStr">
         <is>
@@ -12194,7 +12194,7 @@
         <v>728</v>
       </c>
       <c r="X240" s="4" t="n">
-        <v>3</v>
+        <v>58</v>
       </c>
       <c r="Y240" s="4" t="inlineStr">
         <is>
@@ -12235,7 +12235,7 @@
         <v>744</v>
       </c>
       <c r="X241" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Y241" s="7" t="inlineStr">
         <is>
@@ -12276,7 +12276,7 @@
         <v>786</v>
       </c>
       <c r="X242" s="4" t="n">
-        <v>1</v>
+        <v>70</v>
       </c>
       <c r="Y242" s="4" t="inlineStr">
         <is>
@@ -12317,7 +12317,7 @@
         <v>769</v>
       </c>
       <c r="X243" s="7" t="n">
-        <v>70</v>
+        <v>5</v>
       </c>
       <c r="Y243" s="7" t="inlineStr">
         <is>
@@ -12412,7 +12412,7 @@
         </is>
       </c>
       <c r="AB245" s="7" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="AC245" s="7" t="inlineStr">
         <is>
@@ -12453,7 +12453,7 @@
         </is>
       </c>
       <c r="AB246" s="4" t="n">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="AC246" s="4" t="inlineStr">
         <is>
@@ -12481,7 +12481,7 @@
         <v>728</v>
       </c>
       <c r="X247" s="7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="Y247" s="7" t="inlineStr">
         <is>
@@ -12494,7 +12494,7 @@
         </is>
       </c>
       <c r="AB247" s="7" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="AC247" s="7" t="inlineStr">
         <is>
@@ -12522,7 +12522,7 @@
         <v>709</v>
       </c>
       <c r="X248" s="4" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Y248" s="4" t="inlineStr">
         <is>
@@ -12604,7 +12604,7 @@
         <v>735</v>
       </c>
       <c r="X250" s="4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="Y250" s="4" t="inlineStr">
         <is>
@@ -12645,7 +12645,7 @@
         <v>773</v>
       </c>
       <c r="X251" s="7" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="Y251" s="7" t="inlineStr">
         <is>
@@ -12686,7 +12686,7 @@
         <v>2142</v>
       </c>
       <c r="X252" s="4" t="n">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="Y252" s="4" t="inlineStr">
         <is>
@@ -12727,7 +12727,7 @@
         <v>2408</v>
       </c>
       <c r="X253" s="7" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="Y253" s="7" t="inlineStr">
         <is>
@@ -12768,7 +12768,7 @@
         <v>2141</v>
       </c>
       <c r="X254" s="4" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="Y254" s="4" t="inlineStr">
         <is>
@@ -12781,7 +12781,7 @@
         </is>
       </c>
       <c r="AB254" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AC254" s="4" t="inlineStr">
         <is>
@@ -12822,7 +12822,7 @@
         </is>
       </c>
       <c r="AB255" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AC255" s="7" t="inlineStr">
         <is>
@@ -12945,7 +12945,7 @@
         </is>
       </c>
       <c r="AB258" s="4" t="n">
-        <v>200</v>
+        <v>176</v>
       </c>
       <c r="AC258" s="4" t="inlineStr">
         <is>
@@ -12986,7 +12986,7 @@
         </is>
       </c>
       <c r="AB259" s="7" t="n">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="AC259" s="7" t="inlineStr">
         <is>
@@ -13014,7 +13014,7 @@
         <v>2265</v>
       </c>
       <c r="X260" s="4" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="Y260" s="4" t="inlineStr">
         <is>
@@ -13055,7 +13055,7 @@
         <v>2187</v>
       </c>
       <c r="X261" s="7" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="Y261" s="7" t="inlineStr">
         <is>
@@ -13096,7 +13096,7 @@
         <v>2127</v>
       </c>
       <c r="X262" s="4" t="n">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="Y262" s="4" t="inlineStr">
         <is>
@@ -13137,7 +13137,7 @@
         <v>2022</v>
       </c>
       <c r="X263" s="7" t="n">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="Y263" s="7" t="inlineStr">
         <is>
@@ -13178,7 +13178,7 @@
         <v>2040</v>
       </c>
       <c r="X264" s="4" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="Y264" s="4" t="inlineStr">
         <is>
@@ -13232,7 +13232,7 @@
         </is>
       </c>
       <c r="AB265" s="7" t="n">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="AC265" s="7" t="inlineStr">
         <is>
@@ -13260,7 +13260,7 @@
         <v>2187</v>
       </c>
       <c r="X266" s="4" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="Y266" s="4" t="inlineStr">
         <is>
@@ -13273,7 +13273,7 @@
         </is>
       </c>
       <c r="AB266" s="4" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="AC266" s="4" t="inlineStr">
         <is>
@@ -13301,20 +13301,20 @@
         <v>2290</v>
       </c>
       <c r="X267" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="Y267" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="Z267" s="7" t="inlineStr">
+        <is>
+          <t>com.logistics.rider.glovo</t>
+        </is>
+      </c>
+      <c r="AB267" s="7" t="n">
         <v>27</v>
-      </c>
-      <c r="Y267" s="7" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="Z267" s="7" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.glovo</t>
-        </is>
-      </c>
-      <c r="AB267" s="7" t="n">
-        <v>59</v>
       </c>
       <c r="AC267" s="7" t="inlineStr">
         <is>
@@ -13355,7 +13355,7 @@
         </is>
       </c>
       <c r="AB268" s="4" t="n">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="AC268" s="4" t="inlineStr">
         <is>
@@ -13396,7 +13396,7 @@
         </is>
       </c>
       <c r="AB269" s="7" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="AC269" s="7" t="inlineStr">
         <is>
@@ -13478,7 +13478,7 @@
         </is>
       </c>
       <c r="AB271" s="7" t="n">
-        <v>6</v>
+        <v>103</v>
       </c>
       <c r="AC271" s="7" t="inlineStr">
         <is>
@@ -13519,7 +13519,7 @@
         </is>
       </c>
       <c r="AB272" s="4" t="n">
-        <v>103</v>
+        <v>6</v>
       </c>
       <c r="AC272" s="4" t="inlineStr">
         <is>
@@ -13547,7 +13547,7 @@
         <v>2160</v>
       </c>
       <c r="X273" s="7" t="n">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="Y273" s="7" t="inlineStr">
         <is>
@@ -13588,7 +13588,7 @@
         <v>2276</v>
       </c>
       <c r="X274" s="4" t="n">
-        <v>61</v>
+        <v>13</v>
       </c>
       <c r="Y274" s="4" t="inlineStr">
         <is>
@@ -13632,7 +13632,7 @@
         </is>
       </c>
       <c r="AB275" s="7" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="AC275" s="7" t="inlineStr">
         <is>
@@ -13650,7 +13650,7 @@
       <c r="U276" s="4" t="n"/>
       <c r="V276" s="4" t="n"/>
       <c r="X276" s="4" t="n">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="Y276" s="4" t="inlineStr">
         <is>
@@ -13663,7 +13663,7 @@
         </is>
       </c>
       <c r="AB276" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="AC276" s="4" t="inlineStr">
         <is>
@@ -13681,7 +13681,7 @@
       <c r="U277" s="7" t="n"/>
       <c r="V277" s="7" t="n"/>
       <c r="X277" s="7" t="n">
-        <v>11</v>
+        <v>57</v>
       </c>
       <c r="Y277" s="7" t="inlineStr">
         <is>
@@ -13712,7 +13712,7 @@
       <c r="U278" s="4" t="n"/>
       <c r="V278" s="4" t="n"/>
       <c r="X278" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Y278" s="4" t="inlineStr">
         <is>
@@ -13743,7 +13743,7 @@
       <c r="U279" s="7" t="n"/>
       <c r="V279" s="7" t="n"/>
       <c r="X279" s="7" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="Y279" s="7" t="inlineStr">
         <is>
@@ -13774,7 +13774,7 @@
       <c r="U280" s="4" t="n"/>
       <c r="V280" s="4" t="n"/>
       <c r="X280" s="4" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="Y280" s="4" t="inlineStr">
         <is>
@@ -13805,7 +13805,7 @@
       <c r="U281" s="7" t="n"/>
       <c r="V281" s="7" t="n"/>
       <c r="X281" s="7" t="n">
-        <v>3</v>
+        <v>52</v>
       </c>
       <c r="Y281" s="7" t="inlineStr">
         <is>
@@ -13836,7 +13836,7 @@
       <c r="U282" s="4" t="n"/>
       <c r="V282" s="4" t="n"/>
       <c r="X282" s="4" t="n">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="Y282" s="4" t="inlineStr">
         <is>
@@ -13942,7 +13942,7 @@
         </is>
       </c>
       <c r="AB285" s="7" t="n">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="AC285" s="7" t="inlineStr">
         <is>
@@ -13960,7 +13960,7 @@
       <c r="U286" s="4" t="n"/>
       <c r="V286" s="4" t="n"/>
       <c r="X286" s="4" t="n">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="Y286" s="4" t="inlineStr">
         <is>
@@ -13973,7 +13973,7 @@
         </is>
       </c>
       <c r="AB286" s="4" t="n">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="AC286" s="4" t="inlineStr">
         <is>
@@ -13991,7 +13991,7 @@
       <c r="U287" s="7" t="n"/>
       <c r="V287" s="7" t="n"/>
       <c r="X287" s="7" t="n">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="Y287" s="7" t="inlineStr">
         <is>
@@ -14004,7 +14004,7 @@
         </is>
       </c>
       <c r="AB287" s="7" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="AC287" s="7" t="inlineStr">
         <is>
@@ -14022,7 +14022,7 @@
       <c r="U288" s="4" t="n"/>
       <c r="V288" s="4" t="n"/>
       <c r="X288" s="4" t="n">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="Y288" s="4" t="inlineStr">
         <is>
@@ -14035,7 +14035,7 @@
         </is>
       </c>
       <c r="AB288" s="4" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="AC288" s="4" t="inlineStr">
         <is>
@@ -14053,7 +14053,7 @@
       <c r="U289" s="7" t="n"/>
       <c r="V289" s="7" t="n"/>
       <c r="X289" s="7" t="n">
-        <v>52</v>
+        <v>1</v>
       </c>
       <c r="Y289" s="7" t="inlineStr">
         <is>
@@ -14221,7 +14221,7 @@
         </is>
       </c>
       <c r="AB294" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="AC294" s="4" t="inlineStr">
         <is>
@@ -14252,7 +14252,7 @@
         </is>
       </c>
       <c r="AB295" s="7" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="AC295" s="7" t="inlineStr">
         <is>
@@ -14301,7 +14301,7 @@
       <c r="U297" s="7" t="n"/>
       <c r="V297" s="7" t="n"/>
       <c r="X297" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Y297" s="7" t="inlineStr">
         <is>
@@ -14332,7 +14332,7 @@
       <c r="U298" s="4" t="n"/>
       <c r="V298" s="4" t="n"/>
       <c r="X298" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Y298" s="4" t="inlineStr">
         <is>
@@ -14345,7 +14345,7 @@
         </is>
       </c>
       <c r="AB298" s="4" t="n">
-        <v>258</v>
+        <v>90</v>
       </c>
       <c r="AC298" s="4" t="inlineStr">
         <is>
@@ -14376,7 +14376,7 @@
         </is>
       </c>
       <c r="AB299" s="7" t="n">
-        <v>90</v>
+        <v>258</v>
       </c>
       <c r="AC299" s="7" t="inlineStr">
         <is>
@@ -14469,7 +14469,7 @@
         </is>
       </c>
       <c r="AB302" s="4" t="n">
-        <v>141</v>
+        <v>1</v>
       </c>
       <c r="AC302" s="4" t="inlineStr">
         <is>
@@ -14487,7 +14487,7 @@
       <c r="U303" s="7" t="n"/>
       <c r="V303" s="7" t="n"/>
       <c r="X303" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Y303" s="7" t="inlineStr">
         <is>
@@ -14500,7 +14500,7 @@
         </is>
       </c>
       <c r="AB303" s="7" t="n">
-        <v>1</v>
+        <v>141</v>
       </c>
       <c r="AC303" s="7" t="inlineStr">
         <is>
@@ -14518,7 +14518,7 @@
       <c r="U304" s="4" t="n"/>
       <c r="V304" s="4" t="n"/>
       <c r="X304" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="Y304" s="4" t="inlineStr">
         <is>
@@ -14562,7 +14562,7 @@
         </is>
       </c>
       <c r="AB305" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AC305" s="7" t="inlineStr">
         <is>
@@ -14593,7 +14593,7 @@
         </is>
       </c>
       <c r="AB306" s="4" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="AC306" s="4" t="inlineStr">
         <is>
@@ -14624,7 +14624,7 @@
         </is>
       </c>
       <c r="AB307" s="7" t="n">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="AC307" s="7" t="inlineStr">
         <is>
@@ -14642,7 +14642,7 @@
       <c r="U308" s="4" t="n"/>
       <c r="V308" s="4" t="n"/>
       <c r="X308" s="4" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="Y308" s="4" t="inlineStr">
         <is>
@@ -14673,7 +14673,7 @@
       <c r="U309" s="7" t="n"/>
       <c r="V309" s="7" t="n"/>
       <c r="X309" s="7" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="Y309" s="7" t="inlineStr">
         <is>
@@ -14704,7 +14704,7 @@
       <c r="U310" s="4" t="n"/>
       <c r="V310" s="4" t="n"/>
       <c r="X310" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="Y310" s="4" t="inlineStr">
         <is>
@@ -14735,7 +14735,7 @@
       <c r="U311" s="7" t="n"/>
       <c r="V311" s="7" t="n"/>
       <c r="X311" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Y311" s="7" t="inlineStr">
         <is>
@@ -14890,7 +14890,7 @@
       <c r="U316" s="4" t="n"/>
       <c r="V316" s="4" t="n"/>
       <c r="X316" s="4" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Y316" s="4" t="inlineStr">
         <is>
@@ -14921,7 +14921,7 @@
       <c r="U317" s="7" t="n"/>
       <c r="V317" s="7" t="n"/>
       <c r="X317" s="7" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Y317" s="7" t="inlineStr">
         <is>
@@ -14965,7 +14965,7 @@
         </is>
       </c>
       <c r="AB318" s="4" t="n">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="AC318" s="4" t="inlineStr">
         <is>
@@ -14983,7 +14983,7 @@
       <c r="U319" s="7" t="n"/>
       <c r="V319" s="7" t="n"/>
       <c r="X319" s="7" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Y319" s="7" t="inlineStr">
         <is>
@@ -14996,7 +14996,7 @@
         </is>
       </c>
       <c r="AB319" s="7" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="AC319" s="7" t="inlineStr">
         <is>
@@ -15014,7 +15014,7 @@
       <c r="U320" s="4" t="n"/>
       <c r="V320" s="4" t="n"/>
       <c r="X320" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="Y320" s="4" t="inlineStr">
         <is>
@@ -15107,7 +15107,7 @@
       <c r="U323" s="7" t="n"/>
       <c r="V323" s="7" t="n"/>
       <c r="X323" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Y323" s="7" t="inlineStr">
         <is>
@@ -15138,7 +15138,7 @@
       <c r="U324" s="4" t="n"/>
       <c r="V324" s="4" t="n"/>
       <c r="X324" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Y324" s="4" t="inlineStr">
         <is>
@@ -15151,7 +15151,7 @@
         </is>
       </c>
       <c r="AB324" s="4" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="AC324" s="4" t="inlineStr">
         <is>
@@ -15182,7 +15182,7 @@
         </is>
       </c>
       <c r="AB325" s="7" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="AC325" s="7" t="inlineStr">
         <is>
@@ -15244,7 +15244,7 @@
         </is>
       </c>
       <c r="AB327" s="7" t="n">
-        <v>36</v>
+        <v>147</v>
       </c>
       <c r="AC327" s="7" t="inlineStr">
         <is>
@@ -15275,7 +15275,7 @@
         </is>
       </c>
       <c r="AB328" s="4" t="n">
-        <v>147</v>
+        <v>3</v>
       </c>
       <c r="AC328" s="4" t="inlineStr">
         <is>
@@ -15461,7 +15461,7 @@
         </is>
       </c>
       <c r="AB334" s="4" t="n">
-        <v>330</v>
+        <v>70</v>
       </c>
       <c r="AC334" s="4" t="inlineStr">
         <is>
@@ -15492,7 +15492,7 @@
         </is>
       </c>
       <c r="AB335" s="7" t="n">
-        <v>70</v>
+        <v>330</v>
       </c>
       <c r="AC335" s="7" t="inlineStr">
         <is>
@@ -15585,7 +15585,7 @@
         </is>
       </c>
       <c r="AB338" s="4" t="n">
-        <v>22</v>
+        <v>143</v>
       </c>
       <c r="AC338" s="4" t="inlineStr">
         <is>
@@ -15634,7 +15634,7 @@
       <c r="U340" s="4" t="n"/>
       <c r="V340" s="4" t="n"/>
       <c r="X340" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y340" s="4" t="inlineStr">
         <is>
@@ -15647,7 +15647,7 @@
         </is>
       </c>
       <c r="AB340" s="4" t="n">
-        <v>143</v>
+        <v>22</v>
       </c>
       <c r="AC340" s="4" t="inlineStr">
         <is>
@@ -15665,7 +15665,7 @@
       <c r="U341" s="7" t="n"/>
       <c r="V341" s="7" t="n"/>
       <c r="X341" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y341" s="7" t="inlineStr">
         <is>
@@ -15678,7 +15678,7 @@
         </is>
       </c>
       <c r="AB341" s="7" t="n">
-        <v>72</v>
+        <v>2</v>
       </c>
       <c r="AC341" s="7" t="inlineStr">
         <is>
@@ -15709,7 +15709,7 @@
         </is>
       </c>
       <c r="AB342" s="4" t="n">
-        <v>2</v>
+        <v>72</v>
       </c>
       <c r="AC342" s="4" t="inlineStr">
         <is>
@@ -15727,7 +15727,7 @@
       <c r="U343" s="7" t="n"/>
       <c r="V343" s="7" t="n"/>
       <c r="X343" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Y343" s="7" t="inlineStr">
         <is>
@@ -15758,7 +15758,7 @@
       <c r="U344" s="4" t="n"/>
       <c r="V344" s="4" t="n"/>
       <c r="X344" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Y344" s="4" t="inlineStr">
         <is>
@@ -15885,7 +15885,7 @@
       <c r="Y348" s="4" t="n"/>
       <c r="Z348" s="4" t="n"/>
       <c r="AB348" s="4" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="AC348" s="4" t="inlineStr">
         <is>
@@ -15906,7 +15906,7 @@
       <c r="Y349" s="7" t="n"/>
       <c r="Z349" s="7" t="n"/>
       <c r="AB349" s="7" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="AC349" s="7" t="inlineStr">
         <is>
@@ -16074,7 +16074,7 @@
       <c r="Y357" s="7" t="n"/>
       <c r="Z357" s="7" t="n"/>
       <c r="AB357" s="7" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="AC357" s="7" t="inlineStr">
         <is>
@@ -16095,7 +16095,7 @@
       <c r="Y358" s="4" t="n"/>
       <c r="Z358" s="4" t="n"/>
       <c r="AB358" s="4" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="AC358" s="4" t="inlineStr">
         <is>
@@ -16116,7 +16116,7 @@
       <c r="Y359" s="7" t="n"/>
       <c r="Z359" s="7" t="n"/>
       <c r="AB359" s="7" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="AC359" s="7" t="inlineStr">
         <is>
@@ -16137,7 +16137,7 @@
       <c r="Y360" s="4" t="n"/>
       <c r="Z360" s="4" t="n"/>
       <c r="AB360" s="4" t="n">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="AC360" s="4" t="inlineStr">
         <is>
@@ -16326,7 +16326,7 @@
       <c r="Y369" s="7" t="n"/>
       <c r="Z369" s="7" t="n"/>
       <c r="AB369" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="AC369" s="7" t="inlineStr">
         <is>
@@ -16347,7 +16347,7 @@
       <c r="Y370" s="4" t="n"/>
       <c r="Z370" s="4" t="n"/>
       <c r="AB370" s="4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AC370" s="4" t="inlineStr">
         <is>
@@ -16452,7 +16452,7 @@
       <c r="Y375" s="7" t="n"/>
       <c r="Z375" s="7" t="n"/>
       <c r="AB375" s="7" t="n">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="AC375" s="7" t="inlineStr">
         <is>
@@ -16473,7 +16473,7 @@
       <c r="Y376" s="4" t="n"/>
       <c r="Z376" s="4" t="n"/>
       <c r="AB376" s="4" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="AC376" s="4" t="inlineStr">
         <is>
@@ -16578,7 +16578,7 @@
       <c r="Y381" s="7" t="n"/>
       <c r="Z381" s="7" t="n"/>
       <c r="AB381" s="7" t="n">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="AC381" s="7" t="inlineStr">
         <is>
@@ -16599,7 +16599,7 @@
       <c r="Y382" s="4" t="n"/>
       <c r="Z382" s="4" t="n"/>
       <c r="AB382" s="4" t="n">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="AC382" s="4" t="inlineStr">
         <is>
@@ -16641,7 +16641,7 @@
       <c r="Y384" s="4" t="n"/>
       <c r="Z384" s="4" t="n"/>
       <c r="AB384" s="4" t="n">
-        <v>3</v>
+        <v>129</v>
       </c>
       <c r="AC384" s="4" t="inlineStr">
         <is>
@@ -16662,7 +16662,7 @@
       <c r="Y385" s="7" t="n"/>
       <c r="Z385" s="7" t="n"/>
       <c r="AB385" s="7" t="n">
-        <v>129</v>
+        <v>3</v>
       </c>
       <c r="AC385" s="7" t="inlineStr">
         <is>
@@ -16809,7 +16809,7 @@
       <c r="Y392" s="4" t="n"/>
       <c r="Z392" s="4" t="n"/>
       <c r="AB392" s="4" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="AC392" s="4" t="inlineStr">
         <is>
@@ -16830,7 +16830,7 @@
       <c r="Y393" s="7" t="n"/>
       <c r="Z393" s="7" t="n"/>
       <c r="AB393" s="7" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="AC393" s="7" t="inlineStr">
         <is>
@@ -16893,7 +16893,7 @@
       <c r="Y396" s="4" t="n"/>
       <c r="Z396" s="4" t="n"/>
       <c r="AB396" s="4" t="n">
-        <v>1</v>
+        <v>78</v>
       </c>
       <c r="AC396" s="4" t="inlineStr">
         <is>
@@ -16914,7 +16914,7 @@
       <c r="Y397" s="7" t="n"/>
       <c r="Z397" s="7" t="n"/>
       <c r="AB397" s="7" t="n">
-        <v>78</v>
+        <v>1</v>
       </c>
       <c r="AC397" s="7" t="inlineStr">
         <is>
@@ -17292,7 +17292,7 @@
       <c r="Y415" s="7" t="n"/>
       <c r="Z415" s="7" t="n"/>
       <c r="AB415" s="7" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="AC415" s="7" t="inlineStr">
         <is>
@@ -17313,7 +17313,7 @@
       <c r="Y416" s="4" t="n"/>
       <c r="Z416" s="4" t="n"/>
       <c r="AB416" s="4" t="n">
-        <v>22</v>
+        <v>135</v>
       </c>
       <c r="AC416" s="4" t="inlineStr">
         <is>
@@ -17334,7 +17334,7 @@
       <c r="Y417" s="7" t="n"/>
       <c r="Z417" s="7" t="n"/>
       <c r="AB417" s="7" t="n">
-        <v>135</v>
+        <v>1</v>
       </c>
       <c r="AC417" s="7" t="inlineStr">
         <is>
@@ -17376,7 +17376,7 @@
       <c r="Y419" s="7" t="n"/>
       <c r="Z419" s="7" t="n"/>
       <c r="AB419" s="7" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="AC419" s="7" t="inlineStr">
         <is>
@@ -17397,7 +17397,7 @@
       <c r="Y420" s="4" t="n"/>
       <c r="Z420" s="4" t="n"/>
       <c r="AB420" s="4" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="AC420" s="4" t="inlineStr">
         <is>
@@ -17460,7 +17460,7 @@
       <c r="Y423" s="7" t="n"/>
       <c r="Z423" s="7" t="n"/>
       <c r="AB423" s="7" t="n">
-        <v>1</v>
+        <v>289</v>
       </c>
       <c r="AC423" s="7" t="inlineStr">
         <is>
@@ -17481,7 +17481,7 @@
       <c r="Y424" s="4" t="n"/>
       <c r="Z424" s="4" t="n"/>
       <c r="AB424" s="4" t="n">
-        <v>289</v>
+        <v>49</v>
       </c>
       <c r="AC424" s="4" t="inlineStr">
         <is>
@@ -17502,7 +17502,7 @@
       <c r="Y425" s="7" t="n"/>
       <c r="Z425" s="7" t="n"/>
       <c r="AB425" s="7" t="n">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="AC425" s="7" t="inlineStr">
         <is>
@@ -17523,7 +17523,7 @@
       <c r="Y426" s="4" t="n"/>
       <c r="Z426" s="4" t="n"/>
       <c r="AB426" s="4" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="AC426" s="4" t="inlineStr">
         <is>
@@ -17544,7 +17544,7 @@
       <c r="Y427" s="7" t="n"/>
       <c r="Z427" s="7" t="n"/>
       <c r="AB427" s="7" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="AC427" s="7" t="inlineStr">
         <is>
@@ -17565,7 +17565,7 @@
       <c r="Y428" s="4" t="n"/>
       <c r="Z428" s="4" t="n"/>
       <c r="AB428" s="4" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="AC428" s="4" t="inlineStr">
         <is>
@@ -17586,7 +17586,7 @@
       <c r="Y429" s="7" t="n"/>
       <c r="Z429" s="7" t="n"/>
       <c r="AB429" s="7" t="n">
-        <v>16</v>
+        <v>124</v>
       </c>
       <c r="AC429" s="7" t="inlineStr">
         <is>
@@ -17607,7 +17607,7 @@
       <c r="Y430" s="4" t="n"/>
       <c r="Z430" s="4" t="n"/>
       <c r="AB430" s="4" t="n">
-        <v>124</v>
+        <v>2</v>
       </c>
       <c r="AC430" s="4" t="inlineStr">
         <is>
@@ -17628,7 +17628,7 @@
       <c r="Y431" s="7" t="n"/>
       <c r="Z431" s="7" t="n"/>
       <c r="AB431" s="7" t="n">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="AC431" s="7" t="inlineStr">
         <is>
@@ -17649,7 +17649,7 @@
       <c r="Y432" s="4" t="n"/>
       <c r="Z432" s="4" t="n"/>
       <c r="AB432" s="4" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="AC432" s="4" t="inlineStr">
         <is>
@@ -17796,7 +17796,7 @@
       <c r="Y439" s="7" t="n"/>
       <c r="Z439" s="7" t="n"/>
       <c r="AB439" s="7" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="AC439" s="7" t="inlineStr">
         <is>
@@ -17817,7 +17817,7 @@
       <c r="Y440" s="4" t="n"/>
       <c r="Z440" s="4" t="n"/>
       <c r="AB440" s="4" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="AC440" s="4" t="inlineStr">
         <is>
@@ -17838,7 +17838,7 @@
       <c r="Y441" s="7" t="n"/>
       <c r="Z441" s="7" t="n"/>
       <c r="AB441" s="7" t="n">
-        <v>332</v>
+        <v>53</v>
       </c>
       <c r="AC441" s="7" t="inlineStr">
         <is>
@@ -17859,7 +17859,7 @@
       <c r="Y442" s="4" t="n"/>
       <c r="Z442" s="4" t="n"/>
       <c r="AB442" s="4" t="n">
-        <v>53</v>
+        <v>332</v>
       </c>
       <c r="AC442" s="4" t="inlineStr">
         <is>
@@ -17880,7 +17880,7 @@
       <c r="Y443" s="7" t="n"/>
       <c r="Z443" s="7" t="n"/>
       <c r="AB443" s="7" t="n">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="AC443" s="7" t="inlineStr">
         <is>
@@ -17901,7 +17901,7 @@
       <c r="Y444" s="4" t="n"/>
       <c r="Z444" s="4" t="n"/>
       <c r="AB444" s="4" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="AC444" s="4" t="inlineStr">
         <is>
@@ -17964,7 +17964,7 @@
       <c r="Y447" s="7" t="n"/>
       <c r="Z447" s="7" t="n"/>
       <c r="AB447" s="7" t="n">
-        <v>1</v>
+        <v>63</v>
       </c>
       <c r="AC447" s="7" t="inlineStr">
         <is>
@@ -17985,7 +17985,7 @@
       <c r="Y448" s="4" t="n"/>
       <c r="Z448" s="4" t="n"/>
       <c r="AB448" s="4" t="n">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="AC448" s="4" t="inlineStr">
         <is>
@@ -31825,16 +31825,16 @@
         </is>
       </c>
       <c r="AB8" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>com.logistics.rider.efood</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -31903,7 +31903,7 @@
         </is>
       </c>
       <c r="AB9" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
@@ -31912,7 +31912,7 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -31991,7 +31991,7 @@
         </is>
       </c>
       <c r="AB10" t="n">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
@@ -32000,7 +32000,7 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -32078,7 +32078,7 @@
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -32147,7 +32147,7 @@
         </is>
       </c>
       <c r="AB12" t="n">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
@@ -32156,7 +32156,7 @@
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -32225,7 +32225,7 @@
         </is>
       </c>
       <c r="AB13" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
@@ -32234,7 +32234,7 @@
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -32303,16 +32303,16 @@
         </is>
       </c>
       <c r="AB14" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>com.logistics.rider.glovo</t>
+          <t>com.logistics.rider.foodpanda</t>
         </is>
       </c>
     </row>
@@ -32381,7 +32381,7 @@
         </is>
       </c>
       <c r="AB15" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
@@ -32390,7 +32390,7 @@
       </c>
       <c r="AD15" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodpanda</t>
+          <t>com.logistics.rider.foodora</t>
         </is>
       </c>
     </row>
@@ -32459,7 +32459,7 @@
         </is>
       </c>
       <c r="AB16" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
@@ -32468,7 +32468,7 @@
       </c>
       <c r="AD16" t="inlineStr">
         <is>
-          <t>com.logistics.rider.foodora</t>
+          <t>com.logistics.rider.talabat</t>
         </is>
       </c>
     </row>
@@ -32537,7 +32537,7 @@
         </is>
       </c>
       <c r="AB17" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
@@ -32546,7 +32546,7 @@
       </c>
       <c r="AD17" t="inlineStr">
         <is>
-          <t>com.logistics.rider.talabat</t>
+          <t>com.logistics.rider.pedidosya</t>
         </is>
       </c>
     </row>
@@ -32615,7 +32615,7 @@
         </is>
       </c>
       <c r="AB18" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
@@ -32624,7 +32624,7 @@
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>com.logistics.rider.pedidosya</t>
+          <t>com.logistics.rider.hungerstation</t>
         </is>
       </c>
     </row>
@@ -32680,7 +32680,7 @@
         <v>1607</v>
       </c>
       <c r="AB19" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="AC19" t="inlineStr">
         <is>
@@ -32689,7 +32689,7 @@
       </c>
       <c r="AD19" t="inlineStr">
         <is>
-          <t>com.logistics.rider.hungerstation</t>
+          <t>com.logistics.rider.glovo</t>
         </is>
       </c>
     </row>
@@ -32744,19 +32744,6 @@
       <c r="V20" t="n">
         <v>2003</v>
       </c>
-      <c r="AB20" t="n">
-        <v>32</v>
-      </c>
-      <c r="AC20" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="AD20" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.glovo</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="C21" t="inlineStr">
@@ -32808,19 +32795,6 @@
       </c>
       <c r="V21" t="n">
         <v>1</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>3</v>
-      </c>
-      <c r="AC21" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="AD21" t="inlineStr">
-        <is>
-          <t>com.logistics.rider.efood</t>
-        </is>
       </c>
     </row>
     <row r="22">

</xml_diff>